<commit_message>
Elite Only 2020: affichage specifique + chronos vainqueurs
- Tokyo, London, Valencia 2020 marques 'Elite' dans le Excel
- Affichage 'Elite Only' en bleu (#38BDF8) dans le tableau
- Chronos vainqueurs 2020 ajoutes pour ces 3 courses:
  Tokyo 2020: H 2:04:15 (Legese), F 2:17:45 (Salpeter)
  London 2020: H 2:05:41 (Kitata), F 2:18:58 (Kosgei)
  Valencia 2020: H 2:03:00 (Chebet)
- Pris en compte dans Winners Times et records Vue d'ensemble
- Distinction visuelle: Annule=rouge, Elite Only=bleu, Normal=blanc

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$357</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$360</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E357"/>
+  <dimension ref="A1:E360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3574,16 +3574,16 @@
         </is>
       </c>
       <c r="C124" s="3" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>2:04:01</t>
+          <t>2:05:41</t>
         </is>
       </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:18:58</t>
         </is>
       </c>
     </row>
@@ -3599,16 +3599,16 @@
         </is>
       </c>
       <c r="C125" s="5" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D125" s="5" t="inlineStr">
         <is>
-          <t>2:04:39</t>
+          <t>2:04:01</t>
         </is>
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>2:17:26</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -3624,16 +3624,16 @@
         </is>
       </c>
       <c r="C126" s="3" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>2:01:25</t>
+          <t>2:04:39</t>
         </is>
       </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
-          <t>2:18:33</t>
+          <t>2:17:26</t>
         </is>
       </c>
     </row>
@@ -3649,16 +3649,16 @@
         </is>
       </c>
       <c r="C127" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>2:04:01</t>
+          <t>2:01:25</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>2:16:16</t>
+          <t>2:18:33</t>
         </is>
       </c>
     </row>
@@ -3674,23 +3674,23 @@
         </is>
       </c>
       <c r="C128" s="3" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>2:02:27</t>
+          <t>2:04:01</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>2:15:50</t>
+          <t>2:16:16</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>TCS New York City Marathon</t>
+          <t>TCS London Marathon</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
@@ -3699,16 +3699,16 @@
         </is>
       </c>
       <c r="C129" s="5" t="n">
-        <v>2015</v>
+        <v>2025</v>
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>2:10:34</t>
+          <t>2:02:27</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>2:24:25</t>
+          <t>2:15:50</t>
         </is>
       </c>
     </row>
@@ -3724,16 +3724,16 @@
         </is>
       </c>
       <c r="C130" s="3" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>2:07:51</t>
+          <t>2:10:34</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>2:24:26</t>
+          <t>2:24:25</t>
         </is>
       </c>
     </row>
@@ -3749,16 +3749,16 @@
         </is>
       </c>
       <c r="C131" s="5" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>2:10:53</t>
+          <t>2:07:51</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:24:26</t>
         </is>
       </c>
     </row>
@@ -3774,16 +3774,16 @@
         </is>
       </c>
       <c r="C132" s="3" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>2:05:59</t>
+          <t>2:10:53</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>2:22:48</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -3799,16 +3799,16 @@
         </is>
       </c>
       <c r="C133" s="5" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t>2:08:13</t>
+          <t>2:05:59</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>2:22:38</t>
+          <t>2:22:48</t>
         </is>
       </c>
     </row>
@@ -3824,16 +3824,16 @@
         </is>
       </c>
       <c r="C134" s="3" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>2:08:22</t>
+          <t>2:08:13</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
-          <t>2:22:39</t>
+          <t>2:22:38</t>
         </is>
       </c>
     </row>
@@ -3849,16 +3849,16 @@
         </is>
       </c>
       <c r="C135" s="5" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D135" s="5" t="inlineStr">
         <is>
-          <t>2:08:41</t>
+          <t>2:08:22</t>
         </is>
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>2:23:23</t>
+          <t>2:22:39</t>
         </is>
       </c>
     </row>
@@ -3874,16 +3874,16 @@
         </is>
       </c>
       <c r="C136" s="3" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>2:04:58</t>
+          <t>2:08:41</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>2:27:23</t>
+          <t>2:23:23</t>
         </is>
       </c>
     </row>
@@ -3899,16 +3899,16 @@
         </is>
       </c>
       <c r="C137" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D137" s="5" t="inlineStr">
         <is>
-          <t>2:07:39</t>
+          <t>2:04:58</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>2:24:35</t>
+          <t>2:27:23</t>
         </is>
       </c>
     </row>
@@ -3924,23 +3924,23 @@
         </is>
       </c>
       <c r="C138" s="3" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>2:08:09</t>
+          <t>2:07:39</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>2:19:51</t>
+          <t>2:24:35</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>TCS Sydney Marathon presented by ASICS</t>
+          <t>TCS New York City Marathon</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
@@ -3949,16 +3949,16 @@
         </is>
       </c>
       <c r="C139" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>2:08:20</t>
+          <t>2:08:09</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t>2:26:47</t>
+          <t>2:19:51</t>
         </is>
       </c>
     </row>
@@ -3974,16 +3974,16 @@
         </is>
       </c>
       <c r="C140" s="3" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>2:06:17</t>
+          <t>2:08:20</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>2:21:40</t>
+          <t>2:26:47</t>
         </is>
       </c>
     </row>
@@ -3999,23 +3999,23 @@
         </is>
       </c>
       <c r="C141" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>2:06:06</t>
+          <t>2:06:17</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t>2:18:22</t>
+          <t>2:21:40</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>TCS Toronto Waterfront Marathon</t>
+          <t>TCS Sydney Marathon presented by ASICS</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -4024,16 +4024,16 @@
         </is>
       </c>
       <c r="C142" s="3" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>2:09:20</t>
+          <t>2:06:06</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>2:23:11</t>
+          <t>2:18:22</t>
         </is>
       </c>
     </row>
@@ -4049,16 +4049,16 @@
         </is>
       </c>
       <c r="C143" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D143" s="5" t="inlineStr">
         <is>
-          <t>2:07:16</t>
+          <t>2:09:20</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t>2:20:44</t>
+          <t>2:23:11</t>
         </is>
       </c>
     </row>
@@ -4074,23 +4074,23 @@
         </is>
       </c>
       <c r="C144" s="3" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>2:08:05</t>
+          <t>2:07:16</t>
         </is>
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
-          <t>2:21:04</t>
+          <t>2:20:44</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>Taipei Marathon</t>
+          <t>TCS Toronto Waterfront Marathon</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
@@ -4099,16 +4099,16 @@
         </is>
       </c>
       <c r="C145" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D145" s="5" t="inlineStr">
         <is>
-          <t>2:11:05</t>
+          <t>2:08:05</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t>2:27:14</t>
+          <t>2:21:04</t>
         </is>
       </c>
     </row>
@@ -4124,16 +4124,16 @@
         </is>
       </c>
       <c r="C146" s="3" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>2:11:41</t>
+          <t>2:11:05</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>2:32:47</t>
+          <t>2:27:14</t>
         </is>
       </c>
     </row>
@@ -4149,23 +4149,23 @@
         </is>
       </c>
       <c r="C147" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D147" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:11:41</t>
         </is>
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:32:47</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Tata Mumbai Marathon</t>
+          <t>Taipei Marathon</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
@@ -4174,16 +4174,16 @@
         </is>
       </c>
       <c r="C148" s="3" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>2:07:32</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>2:24:15</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -4199,16 +4199,16 @@
         </is>
       </c>
       <c r="C149" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D149" s="5" t="inlineStr">
         <is>
-          <t>2:07:50</t>
+          <t>2:07:32</t>
         </is>
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t>2:26:06</t>
+          <t>2:24:15</t>
         </is>
       </c>
     </row>
@@ -4224,16 +4224,16 @@
         </is>
       </c>
       <c r="C150" s="3" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>2:11:44</t>
+          <t>2:07:50</t>
         </is>
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
-          <t>2:24:56</t>
+          <t>2:26:06</t>
         </is>
       </c>
     </row>
@@ -4249,23 +4249,23 @@
         </is>
       </c>
       <c r="C151" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D151" s="5" t="inlineStr">
         <is>
-          <t>2:09:55</t>
+          <t>2:11:44</t>
         </is>
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t>2:25:13</t>
+          <t>2:24:56</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Tokyo Marathon</t>
+          <t>Tata Mumbai Marathon</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
@@ -4274,16 +4274,16 @@
         </is>
       </c>
       <c r="C152" s="3" t="n">
-        <v>2015</v>
+        <v>2026</v>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>2:06:00</t>
+          <t>2:09:55</t>
         </is>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>2:23:15</t>
+          <t>2:25:13</t>
         </is>
       </c>
     </row>
@@ -4299,16 +4299,16 @@
         </is>
       </c>
       <c r="C153" s="5" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="D153" s="5" t="inlineStr">
         <is>
-          <t>2:06:56</t>
+          <t>2:06:00</t>
         </is>
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t>2:21:27</t>
+          <t>2:23:15</t>
         </is>
       </c>
     </row>
@@ -4324,16 +4324,16 @@
         </is>
       </c>
       <c r="C154" s="3" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>2:03:58</t>
+          <t>2:06:56</t>
         </is>
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:21:27</t>
         </is>
       </c>
     </row>
@@ -4349,16 +4349,16 @@
         </is>
       </c>
       <c r="C155" s="5" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="D155" s="5" t="inlineStr">
         <is>
-          <t>2:05:30</t>
+          <t>2:03:58</t>
         </is>
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>2:19:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -4374,16 +4374,16 @@
         </is>
       </c>
       <c r="C156" s="3" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>2:04:15</t>
+          <t>2:05:30</t>
         </is>
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:19:51</t>
         </is>
       </c>
     </row>
@@ -4399,16 +4399,16 @@
         </is>
       </c>
       <c r="C157" s="5" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="D157" s="5" t="inlineStr">
         <is>
-          <t>2:02:40</t>
+          <t>2:04:15</t>
         </is>
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>2:16:02</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -4424,16 +4424,16 @@
         </is>
       </c>
       <c r="C158" s="3" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>2:05:22</t>
+          <t>2:04:15</t>
         </is>
       </c>
       <c r="E158" s="3" t="inlineStr">
         <is>
-          <t>2:16:28</t>
+          <t>2:17:45</t>
         </is>
       </c>
     </row>
@@ -4449,16 +4449,16 @@
         </is>
       </c>
       <c r="C159" s="5" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D159" s="5" t="inlineStr">
         <is>
-          <t>2:02:16</t>
+          <t>2:02:40</t>
         </is>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
-          <t>2:15:55</t>
+          <t>2:16:02</t>
         </is>
       </c>
     </row>
@@ -4474,16 +4474,16 @@
         </is>
       </c>
       <c r="C160" s="3" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>2:03:23</t>
+          <t>2:05:22</t>
         </is>
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
-          <t>2:16:31</t>
+          <t>2:16:28</t>
         </is>
       </c>
     </row>
@@ -4499,23 +4499,23 @@
         </is>
       </c>
       <c r="C161" s="5" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D161" s="5" t="inlineStr">
         <is>
-          <t>2:03:37</t>
+          <t>2:02:16</t>
         </is>
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
-          <t>2:14:29</t>
+          <t>2:15:55</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Valencia Marathon Trinidad Alfonso Zurich</t>
+          <t>Tokyo Marathon</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -4524,23 +4524,23 @@
         </is>
       </c>
       <c r="C162" s="3" t="n">
-        <v>2015</v>
+        <v>2025</v>
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>2:06:13</t>
+          <t>2:03:23</t>
         </is>
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:16:31</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>Valencia Marathon Trinidad Alfonso Zurich</t>
+          <t>Tokyo Marathon</t>
         </is>
       </c>
       <c r="B163" s="5" t="inlineStr">
@@ -4549,16 +4549,16 @@
         </is>
       </c>
       <c r="C163" s="5" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="D163" s="5" t="inlineStr">
         <is>
-          <t>2:01:53</t>
+          <t>2:03:37</t>
         </is>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>2:14:57</t>
+          <t>2:14:29</t>
         </is>
       </c>
     </row>
@@ -4574,16 +4574,16 @@
         </is>
       </c>
       <c r="C164" s="3" t="n">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>2:01:48</t>
+          <t>2:06:13</t>
         </is>
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>2:15:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -4599,16 +4599,16 @@
         </is>
       </c>
       <c r="C165" s="5" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="D165" s="5" t="inlineStr">
         <is>
-          <t>2:02:05</t>
+          <t>2:03:00</t>
         </is>
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t>2:16:49</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -4624,23 +4624,23 @@
         </is>
       </c>
       <c r="C166" s="3" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>2:02:24</t>
+          <t>2:01:53</t>
         </is>
       </c>
       <c r="E166" s="3" t="inlineStr">
         <is>
-          <t>2:14:00</t>
+          <t>2:14:57</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>Vienna City Marathon</t>
+          <t>Valencia Marathon Trinidad Alfonso Zurich</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
@@ -4649,23 +4649,23 @@
         </is>
       </c>
       <c r="C167" s="5" t="n">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="D167" s="5" t="inlineStr">
         <is>
-          <t>2:07:31</t>
+          <t>2:01:48</t>
         </is>
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>2:30:09</t>
+          <t>2:15:51</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Vienna City Marathon</t>
+          <t>Valencia Marathon Trinidad Alfonso Zurich</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -4674,23 +4674,23 @@
         </is>
       </c>
       <c r="C168" s="3" t="n">
-        <v>2017</v>
+        <v>2024</v>
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>2:08:40</t>
+          <t>2:02:05</t>
         </is>
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
-          <t>2:24:20</t>
+          <t>2:16:49</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>Vienna City Marathon</t>
+          <t>Valencia Marathon Trinidad Alfonso Zurich</t>
         </is>
       </c>
       <c r="B169" s="5" t="inlineStr">
@@ -4699,16 +4699,16 @@
         </is>
       </c>
       <c r="C169" s="5" t="n">
-        <v>2019</v>
+        <v>2025</v>
       </c>
       <c r="D169" s="5" t="inlineStr">
         <is>
-          <t>2:06:56</t>
+          <t>2:02:24</t>
         </is>
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t>2:22:12</t>
+          <t>2:14:00</t>
         </is>
       </c>
     </row>
@@ -4724,16 +4724,16 @@
         </is>
       </c>
       <c r="C170" s="3" t="n">
-        <v>2021</v>
+        <v>2015</v>
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>2:09:25</t>
+          <t>2:07:31</t>
         </is>
       </c>
       <c r="E170" s="3" t="inlineStr">
         <is>
-          <t>2:24:29</t>
+          <t>2:30:09</t>
         </is>
       </c>
     </row>
@@ -4749,16 +4749,16 @@
         </is>
       </c>
       <c r="C171" s="5" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="D171" s="5" t="inlineStr">
         <is>
-          <t>2:06:53</t>
+          <t>2:08:40</t>
         </is>
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>2:20:59</t>
+          <t>2:24:20</t>
         </is>
       </c>
     </row>
@@ -4774,16 +4774,16 @@
         </is>
       </c>
       <c r="C172" s="3" t="n">
-        <v>2023</v>
+        <v>2019</v>
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>2:05:08</t>
+          <t>2:06:56</t>
         </is>
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
-          <t>2:24:12</t>
+          <t>2:22:12</t>
         </is>
       </c>
     </row>
@@ -4799,16 +4799,16 @@
         </is>
       </c>
       <c r="C173" s="5" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D173" s="5" t="inlineStr">
         <is>
-          <t>2:06:35</t>
+          <t>2:09:25</t>
         </is>
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t>2:24:08</t>
+          <t>2:24:29</t>
         </is>
       </c>
     </row>
@@ -4824,23 +4824,23 @@
         </is>
       </c>
       <c r="C174" s="3" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>2:08:28</t>
+          <t>2:06:53</t>
         </is>
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>2:24:14</t>
+          <t>2:20:59</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>Zurich Marató de Barcelona</t>
+          <t>Vienna City Marathon</t>
         </is>
       </c>
       <c r="B175" s="5" t="inlineStr">
@@ -4853,19 +4853,19 @@
       </c>
       <c r="D175" s="5" t="inlineStr">
         <is>
-          <t>2:05:06</t>
+          <t>2:05:08</t>
         </is>
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>2:19:44</t>
+          <t>2:24:12</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Zurich Marató de Barcelona</t>
+          <t>Vienna City Marathon</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -4878,19 +4878,19 @@
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>2:05:01</t>
+          <t>2:06:35</t>
         </is>
       </c>
       <c r="E176" s="3" t="inlineStr">
         <is>
-          <t>2:19:52</t>
+          <t>2:24:08</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>Zurich Marató de Barcelona</t>
+          <t>Vienna City Marathon</t>
         </is>
       </c>
       <c r="B177" s="5" t="inlineStr">
@@ -4903,12 +4903,12 @@
       </c>
       <c r="D177" s="5" t="inlineStr">
         <is>
-          <t>2:04:13</t>
+          <t>2:08:28</t>
         </is>
       </c>
       <c r="E177" s="5" t="inlineStr">
         <is>
-          <t>2:19:33</t>
+          <t>2:24:14</t>
         </is>
       </c>
     </row>
@@ -4924,23 +4924,23 @@
         </is>
       </c>
       <c r="C178" s="3" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>2:04:57</t>
+          <t>2:05:06</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
-          <t>2:10:53</t>
+          <t>2:19:44</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>Zurich Maratón de Sevilla</t>
+          <t>Zurich Marató de Barcelona</t>
         </is>
       </c>
       <c r="B179" s="5" t="inlineStr">
@@ -4949,23 +4949,23 @@
         </is>
       </c>
       <c r="C179" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D179" s="5" t="inlineStr">
         <is>
-          <t>2:04:59</t>
+          <t>2:05:01</t>
         </is>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>2:20:29</t>
+          <t>2:19:52</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Zurich Maratón de Sevilla</t>
+          <t>Zurich Marató de Barcelona</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
@@ -4974,23 +4974,23 @@
         </is>
       </c>
       <c r="C180" s="3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>2:03:27</t>
+          <t>2:04:13</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
-          <t>2:22:13</t>
+          <t>2:19:33</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>Zurich Maratón de Sevilla</t>
+          <t>Zurich Marató de Barcelona</t>
         </is>
       </c>
       <c r="B181" s="5" t="inlineStr">
@@ -4999,16 +4999,16 @@
         </is>
       </c>
       <c r="C181" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D181" s="5" t="inlineStr">
         <is>
-          <t>2:05:15</t>
+          <t>2:04:57</t>
         </is>
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
-          <t>2:22:17</t>
+          <t>2:10:53</t>
         </is>
       </c>
     </row>
@@ -5024,23 +5024,23 @@
         </is>
       </c>
       <c r="C182" s="3" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>2:03:59</t>
+          <t>2:04:59</t>
         </is>
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>2:20:39</t>
+          <t>2:20:29</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid</t>
+          <t>Zurich Maratón de Sevilla</t>
         </is>
       </c>
       <c r="B183" s="5" t="inlineStr">
@@ -5049,23 +5049,23 @@
         </is>
       </c>
       <c r="C183" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D183" s="5" t="inlineStr">
         <is>
-          <t>2:10:29</t>
+          <t>2:03:27</t>
         </is>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
-          <t>2:26:31</t>
+          <t>2:22:13</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid</t>
+          <t>Zurich Maratón de Sevilla</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
@@ -5074,123 +5074,123 @@
         </is>
       </c>
       <c r="C184" s="3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>2:08:05</t>
+          <t>2:05:15</t>
         </is>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>2:26:19</t>
+          <t>2:22:17</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
+          <t>Zurich Maratón de Sevilla</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>42K</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>2:03:59</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>2:20:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
           <t>Zurich Rock 'n' Roll Running Series Madrid</t>
         </is>
       </c>
-      <c r="B185" s="5" t="inlineStr">
-        <is>
-          <t>42K</t>
-        </is>
-      </c>
-      <c r="C185" s="5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D185" s="5" t="inlineStr">
-        <is>
-          <t>2:09:11</t>
-        </is>
-      </c>
-      <c r="E185" s="5" t="inlineStr">
-        <is>
-          <t>2:25:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="6" t="inlineStr">
-        <is>
-          <t>21K de Montréal</t>
-        </is>
-      </c>
-      <c r="B186" s="7" t="inlineStr">
-        <is>
-          <t>21K</t>
-        </is>
-      </c>
-      <c r="C186" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D186" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E186" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>42K</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>2:10:29</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>2:26:31</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great Bristol Run</t>
+          <t>Zurich Rock 'n' Roll Running Series Madrid</t>
         </is>
       </c>
       <c r="B187" s="5" t="inlineStr">
         <is>
-          <t>21K</t>
+          <t>42K</t>
         </is>
       </c>
       <c r="C187" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D187" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:08:05</t>
         </is>
       </c>
       <c r="E187" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2:26:19</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="6" t="inlineStr">
-        <is>
-          <t>AJ Bell Great Manchester Run</t>
-        </is>
-      </c>
-      <c r="B188" s="7" t="inlineStr">
-        <is>
-          <t>21K</t>
-        </is>
-      </c>
-      <c r="C188" s="7" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D188" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E188" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Zurich Rock 'n' Roll Running Series Madrid</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>42K</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>2:09:11</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>2:25:55</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great North Run</t>
+          <t>21K de Montréal</t>
         </is>
       </c>
       <c r="B189" s="5" t="inlineStr">
@@ -5203,19 +5203,19 @@
       </c>
       <c r="D189" s="5" t="inlineStr">
         <is>
-          <t>1:00:52</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
-          <t>1:09:32</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="6" t="inlineStr">
         <is>
-          <t>Aramco Houston Half Marathon</t>
+          <t>AJ Bell Great Bristol Run</t>
         </is>
       </c>
       <c r="B190" s="7" t="inlineStr">
@@ -5224,23 +5224,23 @@
         </is>
       </c>
       <c r="C190" s="7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D190" s="7" t="inlineStr">
         <is>
-          <t>1:00:42</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>1:04:37</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>Aramco Houston Half Marathon</t>
+          <t>AJ Bell Great Manchester Run</t>
         </is>
       </c>
       <c r="B191" s="5" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="D191" s="5" t="inlineStr">
         <is>
-          <t>0:59:17</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E191" s="5" t="inlineStr">
@@ -5265,7 +5265,7 @@
     <row r="192">
       <c r="A192" s="6" t="inlineStr">
         <is>
-          <t>Aramco Houston Half Marathon</t>
+          <t>AJ Bell Great North Run</t>
         </is>
       </c>
       <c r="B192" s="7" t="inlineStr">
@@ -5274,23 +5274,23 @@
         </is>
       </c>
       <c r="C192" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D192" s="7" t="inlineStr">
         <is>
-          <t>0:59:01</t>
+          <t>1:00:52</t>
         </is>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>1:04:49</t>
+          <t>1:09:32</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>Asics Run Melbourne</t>
+          <t>Aramco Houston Half Marathon</t>
         </is>
       </c>
       <c r="B193" s="5" t="inlineStr">
@@ -5299,23 +5299,23 @@
         </is>
       </c>
       <c r="C193" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D193" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:00:42</t>
         </is>
       </c>
       <c r="E193" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:37</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="6" t="inlineStr">
         <is>
-          <t>Bangsaen21</t>
+          <t>Aramco Houston Half Marathon</t>
         </is>
       </c>
       <c r="B194" s="7" t="inlineStr">
@@ -5324,11 +5324,11 @@
         </is>
       </c>
       <c r="C194" s="7" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D194" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:17</t>
         </is>
       </c>
       <c r="E194" s="7" t="inlineStr">
@@ -5340,7 +5340,7 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>Bangsaen21</t>
+          <t>Aramco Houston Half Marathon</t>
         </is>
       </c>
       <c r="B195" s="5" t="inlineStr">
@@ -5349,23 +5349,23 @@
         </is>
       </c>
       <c r="C195" s="5" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D195" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:01</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:49</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="6" t="inlineStr">
         <is>
-          <t>Bangsaen21</t>
+          <t>Asics Run Melbourne</t>
         </is>
       </c>
       <c r="B196" s="7" t="inlineStr">
@@ -5390,7 +5390,7 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>Brølløbet - The Bridge Run</t>
+          <t>Bangsaen21</t>
         </is>
       </c>
       <c r="B197" s="5" t="inlineStr">
@@ -5399,7 +5399,7 @@
         </is>
       </c>
       <c r="C197" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D197" s="5" t="inlineStr">
         <is>
@@ -5415,7 +5415,7 @@
     <row r="198">
       <c r="A198" s="6" t="inlineStr">
         <is>
-          <t>Burj2Burj Half Marathon</t>
+          <t>Bangsaen21</t>
         </is>
       </c>
       <c r="B198" s="7" t="inlineStr">
@@ -5440,7 +5440,7 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>Burj2Burj Half Marathon</t>
+          <t>Bangsaen21</t>
         </is>
       </c>
       <c r="B199" s="5" t="inlineStr">
@@ -5465,7 +5465,7 @@
     <row r="200">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>Burj2Burj Half Marathon</t>
+          <t>Brølløbet - The Bridge Run</t>
         </is>
       </c>
       <c r="B200" s="7" t="inlineStr">
@@ -5474,23 +5474,23 @@
         </is>
       </c>
       <c r="C200" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D200" s="7" t="inlineStr">
         <is>
-          <t>0:59:26</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>1:06:57</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>Cardiff Half Marathon</t>
+          <t>Burj2Burj Half Marathon</t>
         </is>
       </c>
       <c r="B201" s="5" t="inlineStr">
@@ -5499,7 +5499,7 @@
         </is>
       </c>
       <c r="C201" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D201" s="5" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
     <row r="202">
       <c r="A202" s="6" t="inlineStr">
         <is>
-          <t>Coelmo Napoli City Half Marathon</t>
+          <t>Burj2Burj Half Marathon</t>
         </is>
       </c>
       <c r="B202" s="7" t="inlineStr">
@@ -5540,7 +5540,7 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>Coelmo Napoli City Half Marathon</t>
+          <t>Burj2Burj Half Marathon</t>
         </is>
       </c>
       <c r="B203" s="5" t="inlineStr">
@@ -5553,19 +5553,19 @@
       </c>
       <c r="D203" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:26</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:57</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="6" t="inlineStr">
         <is>
-          <t>Copenhagen Half Marathon</t>
+          <t>Cardiff Half Marathon</t>
         </is>
       </c>
       <c r="B204" s="7" t="inlineStr">
@@ -5574,23 +5574,23 @@
         </is>
       </c>
       <c r="C204" s="7" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D204" s="7" t="inlineStr">
         <is>
-          <t>0:59:11</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E204" s="7" t="inlineStr">
         <is>
-          <t>1:05:53</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>Copenhagen Half Marathon</t>
+          <t>Coelmo Napoli City Half Marathon</t>
         </is>
       </c>
       <c r="B205" s="5" t="inlineStr">
@@ -5599,23 +5599,23 @@
         </is>
       </c>
       <c r="C205" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D205" s="5" t="inlineStr">
         <is>
-          <t>0:58:05</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E205" s="5" t="inlineStr">
         <is>
-          <t>1:05:11</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="6" t="inlineStr">
         <is>
-          <t>Copenhagen Half Marathon</t>
+          <t>Coelmo Napoli City Half Marathon</t>
         </is>
       </c>
       <c r="B206" s="7" t="inlineStr">
@@ -5624,23 +5624,23 @@
         </is>
       </c>
       <c r="C206" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D206" s="7" t="inlineStr">
         <is>
-          <t>0:58:23</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E206" s="7" t="inlineStr">
         <is>
-          <t>1:04:44</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>Disney Princess Half Marathon</t>
+          <t>Copenhagen Half Marathon</t>
         </is>
       </c>
       <c r="B207" s="5" t="inlineStr">
@@ -5649,23 +5649,23 @@
         </is>
       </c>
       <c r="C207" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D207" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:11</t>
         </is>
       </c>
       <c r="E207" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:05:53</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="6" t="inlineStr">
         <is>
-          <t>Disney Princess Half Marathon</t>
+          <t>Copenhagen Half Marathon</t>
         </is>
       </c>
       <c r="B208" s="7" t="inlineStr">
@@ -5674,23 +5674,23 @@
         </is>
       </c>
       <c r="C208" s="7" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D208" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:58:05</t>
         </is>
       </c>
       <c r="E208" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:05:11</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>EDP Lisboa Meia Maratona</t>
+          <t>Copenhagen Half Marathon</t>
         </is>
       </c>
       <c r="B209" s="5" t="inlineStr">
@@ -5699,23 +5699,23 @@
         </is>
       </c>
       <c r="C209" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D209" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:58:23</t>
         </is>
       </c>
       <c r="E209" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:44</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="6" t="inlineStr">
         <is>
-          <t>EDP Lisboa Meia Maratona</t>
+          <t>Disney Princess Half Marathon</t>
         </is>
       </c>
       <c r="B210" s="7" t="inlineStr">
@@ -5740,7 +5740,7 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>EDP Lisboa Meia Maratona</t>
+          <t>Disney Princess Half Marathon</t>
         </is>
       </c>
       <c r="B211" s="5" t="inlineStr">
@@ -5765,7 +5765,7 @@
     <row r="212">
       <c r="A212" s="6" t="inlineStr">
         <is>
-          <t>Eurospin RomaOstia Half Marathon</t>
+          <t>EDP Lisboa Meia Maratona</t>
         </is>
       </c>
       <c r="B212" s="7" t="inlineStr">
@@ -5774,23 +5774,23 @@
         </is>
       </c>
       <c r="C212" s="7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D212" s="7" t="inlineStr">
         <is>
-          <t>0:59:17</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E212" s="7" t="inlineStr">
         <is>
-          <t>1:06:21</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>Eurospin RomaOstia Half Marathon</t>
+          <t>EDP Lisboa Meia Maratona</t>
         </is>
       </c>
       <c r="B213" s="5" t="inlineStr">
@@ -5799,23 +5799,23 @@
         </is>
       </c>
       <c r="C213" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D213" s="5" t="inlineStr">
         <is>
-          <t>1:01:10</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E213" s="5" t="inlineStr">
         <is>
-          <t>1:07:38</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="6" t="inlineStr">
         <is>
-          <t>Eurospin RomaOstia Half Marathon</t>
+          <t>EDP Lisboa Meia Maratona</t>
         </is>
       </c>
       <c r="B214" s="7" t="inlineStr">
@@ -5824,16 +5824,16 @@
         </is>
       </c>
       <c r="C214" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D214" s="7" t="inlineStr">
         <is>
-          <t>0:58:49</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E214" s="7" t="inlineStr">
         <is>
-          <t>1:08:20</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -5849,23 +5849,23 @@
         </is>
       </c>
       <c r="C215" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D215" s="5" t="inlineStr">
         <is>
-          <t>0:58:00</t>
+          <t>0:59:17</t>
         </is>
       </c>
       <c r="E215" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:21</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="6" t="inlineStr">
         <is>
-          <t>Generali Berlin Half Marathon</t>
+          <t>Eurospin RomaOstia Half Marathon</t>
         </is>
       </c>
       <c r="B216" s="7" t="inlineStr">
@@ -5874,23 +5874,23 @@
         </is>
       </c>
       <c r="C216" s="7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D216" s="7" t="inlineStr">
         <is>
-          <t>0:59:01</t>
+          <t>1:01:10</t>
         </is>
       </c>
       <c r="E216" s="7" t="inlineStr">
         <is>
-          <t>1:05:43</t>
+          <t>1:07:38</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>Generali Berlin Half Marathon</t>
+          <t>Eurospin RomaOstia Half Marathon</t>
         </is>
       </c>
       <c r="B217" s="5" t="inlineStr">
@@ -5899,23 +5899,23 @@
         </is>
       </c>
       <c r="C217" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D217" s="5" t="inlineStr">
         <is>
-          <t>0:59:30</t>
+          <t>0:58:49</t>
         </is>
       </c>
       <c r="E217" s="5" t="inlineStr">
         <is>
-          <t>1:06:53</t>
+          <t>1:08:20</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="6" t="inlineStr">
         <is>
-          <t>Generali Berlin Half Marathon</t>
+          <t>Eurospin RomaOstia Half Marathon</t>
         </is>
       </c>
       <c r="B218" s="7" t="inlineStr">
@@ -5924,23 +5924,23 @@
         </is>
       </c>
       <c r="C218" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D218" s="7" t="inlineStr">
         <is>
-          <t>0:58:43</t>
+          <t>0:58:00</t>
         </is>
       </c>
       <c r="E218" s="7" t="inlineStr">
         <is>
-          <t>1:03:35</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>Generali Prague Half Marathon</t>
+          <t>Generali Berlin Half Marathon</t>
         </is>
       </c>
       <c r="B219" s="5" t="inlineStr">
@@ -5953,19 +5953,19 @@
       </c>
       <c r="D219" s="5" t="inlineStr">
         <is>
-          <t>0:59:43</t>
+          <t>0:59:01</t>
         </is>
       </c>
       <c r="E219" s="5" t="inlineStr">
         <is>
-          <t>1:06:00</t>
+          <t>1:05:43</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="6" t="inlineStr">
         <is>
-          <t>Generali Prague Half Marathon</t>
+          <t>Generali Berlin Half Marathon</t>
         </is>
       </c>
       <c r="B220" s="7" t="inlineStr">
@@ -5978,19 +5978,19 @@
       </c>
       <c r="D220" s="7" t="inlineStr">
         <is>
-          <t>0:58:24</t>
+          <t>0:59:30</t>
         </is>
       </c>
       <c r="E220" s="7" t="inlineStr">
         <is>
-          <t>1:08:10</t>
+          <t>1:06:53</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>Generali Prague Half Marathon</t>
+          <t>Generali Berlin Half Marathon</t>
         </is>
       </c>
       <c r="B221" s="5" t="inlineStr">
@@ -6003,19 +6003,19 @@
       </c>
       <c r="D221" s="5" t="inlineStr">
         <is>
-          <t>0:58:54</t>
+          <t>0:58:43</t>
         </is>
       </c>
       <c r="E221" s="5" t="inlineStr">
         <is>
-          <t>1:05:27</t>
+          <t>1:03:35</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="6" t="inlineStr">
         <is>
-          <t>GetPro Bath Half</t>
+          <t>Generali Prague Half Marathon</t>
         </is>
       </c>
       <c r="B222" s="7" t="inlineStr">
@@ -6024,23 +6024,23 @@
         </is>
       </c>
       <c r="C222" s="7" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D222" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:43</t>
         </is>
       </c>
       <c r="E222" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:00</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>GetPro Bath Half</t>
+          <t>Generali Prague Half Marathon</t>
         </is>
       </c>
       <c r="B223" s="5" t="inlineStr">
@@ -6049,23 +6049,23 @@
         </is>
       </c>
       <c r="C223" s="5" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D223" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:58:24</t>
         </is>
       </c>
       <c r="E223" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:08:10</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="6" t="inlineStr">
         <is>
-          <t>Göteborgsvarvet</t>
+          <t>Generali Prague Half Marathon</t>
         </is>
       </c>
       <c r="B224" s="7" t="inlineStr">
@@ -6074,23 +6074,23 @@
         </is>
       </c>
       <c r="C224" s="7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D224" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:58:54</t>
         </is>
       </c>
       <c r="E224" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:05:27</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>Göteborgsvarvet</t>
+          <t>GetPro Bath Half</t>
         </is>
       </c>
       <c r="B225" s="5" t="inlineStr">
@@ -6115,7 +6115,7 @@
     <row r="226">
       <c r="A226" s="6" t="inlineStr">
         <is>
-          <t>HOKA Semi de Paris</t>
+          <t>GetPro Bath Half</t>
         </is>
       </c>
       <c r="B226" s="7" t="inlineStr">
@@ -6124,23 +6124,23 @@
         </is>
       </c>
       <c r="C226" s="7" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D226" s="7" t="inlineStr">
         <is>
-          <t>0:59:38</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E226" s="7" t="inlineStr">
         <is>
-          <t>1:06:01</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>HOKA Semi de Paris</t>
+          <t>Göteborgsvarvet</t>
         </is>
       </c>
       <c r="B227" s="5" t="inlineStr">
@@ -6153,19 +6153,19 @@
       </c>
       <c r="D227" s="5" t="inlineStr">
         <is>
-          <t>1:00:45</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E227" s="5" t="inlineStr">
         <is>
-          <t>1:06:58</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="6" t="inlineStr">
         <is>
-          <t>HOKA Semi de Paris</t>
+          <t>Göteborgsvarvet</t>
         </is>
       </c>
       <c r="B228" s="7" t="inlineStr">
@@ -6178,12 +6178,12 @@
       </c>
       <c r="D228" s="7" t="inlineStr">
         <is>
-          <t>1:00:16</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E228" s="7" t="inlineStr">
         <is>
-          <t>1:07:14</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -6199,23 +6199,23 @@
         </is>
       </c>
       <c r="C229" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D229" s="5" t="inlineStr">
         <is>
-          <t>1:00:11</t>
+          <t>0:59:38</t>
         </is>
       </c>
       <c r="E229" s="5" t="inlineStr">
         <is>
-          <t>1:05:12</t>
+          <t>1:06:01</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="6" t="inlineStr">
         <is>
-          <t>Half Marathon Munchen by Brooks</t>
+          <t>HOKA Semi de Paris</t>
         </is>
       </c>
       <c r="B230" s="7" t="inlineStr">
@@ -6224,23 +6224,23 @@
         </is>
       </c>
       <c r="C230" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D230" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:00:45</t>
         </is>
       </c>
       <c r="E230" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:58</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>Hoka Runaway Sydney Half Marathon</t>
+          <t>HOKA Semi de Paris</t>
         </is>
       </c>
       <c r="B231" s="5" t="inlineStr">
@@ -6253,19 +6253,19 @@
       </c>
       <c r="D231" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:00:16</t>
         </is>
       </c>
       <c r="E231" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:07:14</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="6" t="inlineStr">
         <is>
-          <t>Hyundai Meia Maratona</t>
+          <t>HOKA Semi de Paris</t>
         </is>
       </c>
       <c r="B232" s="7" t="inlineStr">
@@ -6274,23 +6274,23 @@
         </is>
       </c>
       <c r="C232" s="7" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D232" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:00:11</t>
         </is>
       </c>
       <c r="E232" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:05:12</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>Hyundai Meia Maratona</t>
+          <t>Half Marathon Munchen by Brooks</t>
         </is>
       </c>
       <c r="B233" s="5" t="inlineStr">
@@ -6299,7 +6299,7 @@
         </is>
       </c>
       <c r="C233" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D233" s="5" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
     <row r="234">
       <c r="A234" s="6" t="inlineStr">
         <is>
-          <t>Hyundai Meia Maratona</t>
+          <t>Hoka Runaway Sydney Half Marathon</t>
         </is>
       </c>
       <c r="B234" s="7" t="inlineStr">
@@ -6340,7 +6340,7 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>IU Health 500 Festival Mini-Marathon</t>
+          <t>Hyundai Meia Maratona</t>
         </is>
       </c>
       <c r="B235" s="5" t="inlineStr">
@@ -6349,7 +6349,7 @@
         </is>
       </c>
       <c r="C235" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D235" s="5" t="inlineStr">
         <is>
@@ -6365,7 +6365,7 @@
     <row r="236">
       <c r="A236" s="6" t="inlineStr">
         <is>
-          <t>Kagawa Marugame International Half Marathon</t>
+          <t>Hyundai Meia Maratona</t>
         </is>
       </c>
       <c r="B236" s="7" t="inlineStr">
@@ -6374,7 +6374,7 @@
         </is>
       </c>
       <c r="C236" s="7" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D236" s="7" t="inlineStr">
         <is>
@@ -6390,7 +6390,7 @@
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>Life Time Chicago Half Marathon &amp; 5K</t>
+          <t>Hyundai Meia Maratona</t>
         </is>
       </c>
       <c r="B237" s="5" t="inlineStr">
@@ -6399,7 +6399,7 @@
         </is>
       </c>
       <c r="C237" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D237" s="5" t="inlineStr">
         <is>
@@ -6415,7 +6415,7 @@
     <row r="238">
       <c r="A238" s="6" t="inlineStr">
         <is>
-          <t>Life Time Chicago Half Marathon &amp; 5K</t>
+          <t>IU Health 500 Festival Mini-Marathon</t>
         </is>
       </c>
       <c r="B238" s="7" t="inlineStr">
@@ -6440,7 +6440,7 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>London Landmarks Half Marathon</t>
+          <t>Kagawa Marugame International Half Marathon</t>
         </is>
       </c>
       <c r="B239" s="5" t="inlineStr">
@@ -6449,7 +6449,7 @@
         </is>
       </c>
       <c r="C239" s="5" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D239" s="5" t="inlineStr">
         <is>
@@ -6465,7 +6465,7 @@
     <row r="240">
       <c r="A240" s="6" t="inlineStr">
         <is>
-          <t>London Landmarks Half Marathon</t>
+          <t>Life Time Chicago Half Marathon &amp; 5K</t>
         </is>
       </c>
       <c r="B240" s="7" t="inlineStr">
@@ -6474,7 +6474,7 @@
         </is>
       </c>
       <c r="C240" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D240" s="7" t="inlineStr">
         <is>
@@ -6490,7 +6490,7 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>Manchester Half Marathon</t>
+          <t>Life Time Chicago Half Marathon &amp; 5K</t>
         </is>
       </c>
       <c r="B241" s="5" t="inlineStr">
@@ -6515,7 +6515,7 @@
     <row r="242">
       <c r="A242" s="6" t="inlineStr">
         <is>
-          <t>Media Maraton de Bogota</t>
+          <t>London Landmarks Half Marathon</t>
         </is>
       </c>
       <c r="B242" s="7" t="inlineStr">
@@ -6524,7 +6524,7 @@
         </is>
       </c>
       <c r="C242" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D242" s="7" t="inlineStr">
         <is>
@@ -6540,7 +6540,7 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>Medio Maraton de Sevilla</t>
+          <t>London Landmarks Half Marathon</t>
         </is>
       </c>
       <c r="B243" s="5" t="inlineStr">
@@ -6549,23 +6549,23 @@
         </is>
       </c>
       <c r="C243" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D243" s="5" t="inlineStr">
         <is>
-          <t>0:59:21</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E243" s="5" t="inlineStr">
         <is>
-          <t>1:07:59</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="6" t="inlineStr">
         <is>
-          <t>Medio Maraton de Sevilla</t>
+          <t>Manchester Half Marathon</t>
         </is>
       </c>
       <c r="B244" s="7" t="inlineStr">
@@ -6578,19 +6578,19 @@
       </c>
       <c r="D244" s="7" t="inlineStr">
         <is>
-          <t>0:59:33</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E244" s="7" t="inlineStr">
         <is>
-          <t>1:07:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>Medio Maraton de Sevilla</t>
+          <t>Media Maraton de Bogota</t>
         </is>
       </c>
       <c r="B245" s="5" t="inlineStr">
@@ -6599,23 +6599,23 @@
         </is>
       </c>
       <c r="C245" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D245" s="5" t="inlineStr">
         <is>
-          <t>1:00:24</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E245" s="5" t="inlineStr">
         <is>
-          <t>1:06:33</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="inlineStr">
         <is>
-          <t>Mitja Marato Barcelona by Brooks</t>
+          <t>Medio Maraton de Sevilla</t>
         </is>
       </c>
       <c r="B246" s="7" t="inlineStr">
@@ -6624,23 +6624,23 @@
         </is>
       </c>
       <c r="C246" s="7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D246" s="7" t="inlineStr">
         <is>
-          <t>0:58:53</t>
+          <t>0:59:21</t>
         </is>
       </c>
       <c r="E246" s="7" t="inlineStr">
         <is>
-          <t>1:04:37</t>
+          <t>1:07:59</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>Mitja Marato Barcelona by Brooks</t>
+          <t>Medio Maraton de Sevilla</t>
         </is>
       </c>
       <c r="B247" s="5" t="inlineStr">
@@ -6649,23 +6649,23 @@
         </is>
       </c>
       <c r="C247" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D247" s="5" t="inlineStr">
         <is>
-          <t>0:59:21</t>
+          <t>0:59:33</t>
         </is>
       </c>
       <c r="E247" s="5" t="inlineStr">
         <is>
-          <t>1:04:28</t>
+          <t>1:07:18</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="6" t="inlineStr">
         <is>
-          <t>Mitja Marato Barcelona by Brooks</t>
+          <t>Medio Maraton de Sevilla</t>
         </is>
       </c>
       <c r="B248" s="7" t="inlineStr">
@@ -6674,16 +6674,16 @@
         </is>
       </c>
       <c r="C248" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D248" s="7" t="inlineStr">
         <is>
-          <t>0:56:42</t>
+          <t>1:00:24</t>
         </is>
       </c>
       <c r="E248" s="7" t="inlineStr">
         <is>
-          <t>1:04:11</t>
+          <t>1:06:33</t>
         </is>
       </c>
     </row>
@@ -6699,23 +6699,23 @@
         </is>
       </c>
       <c r="C249" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D249" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:58:53</t>
         </is>
       </c>
       <c r="E249" s="5" t="inlineStr">
         <is>
-          <t>1:04:00</t>
+          <t>1:04:37</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="6" t="inlineStr">
         <is>
-          <t>Movistar Madrid Medio Maraton</t>
+          <t>Mitja Marato Barcelona by Brooks</t>
         </is>
       </c>
       <c r="B250" s="7" t="inlineStr">
@@ -6724,23 +6724,23 @@
         </is>
       </c>
       <c r="C250" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D250" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:21</t>
         </is>
       </c>
       <c r="E250" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:28</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>NN CPC Loop Den Haag - Half Marathon</t>
+          <t>Mitja Marato Barcelona by Brooks</t>
         </is>
       </c>
       <c r="B251" s="5" t="inlineStr">
@@ -6753,19 +6753,19 @@
       </c>
       <c r="D251" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:56:42</t>
         </is>
       </c>
       <c r="E251" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:11</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="6" t="inlineStr">
         <is>
-          <t>NN CPC Loop Den Haag - Half Marathon</t>
+          <t>Mitja Marato Barcelona by Brooks</t>
         </is>
       </c>
       <c r="B252" s="7" t="inlineStr">
@@ -6783,14 +6783,14 @@
       </c>
       <c r="E252" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:00</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>NYCRUNS Brooklyn Experience Half Marathon</t>
+          <t>Movistar Madrid Medio Maraton</t>
         </is>
       </c>
       <c r="B253" s="5" t="inlineStr">
@@ -6815,7 +6815,7 @@
     <row r="254">
       <c r="A254" s="6" t="inlineStr">
         <is>
-          <t>NYRR RBC Brooklyn Half</t>
+          <t>NN CPC Loop Den Haag - Half Marathon</t>
         </is>
       </c>
       <c r="B254" s="7" t="inlineStr">
@@ -6840,7 +6840,7 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>Nike Melbourne Marathon Festival</t>
+          <t>NN CPC Loop Den Haag - Half Marathon</t>
         </is>
       </c>
       <c r="B255" s="5" t="inlineStr">
@@ -6849,7 +6849,7 @@
         </is>
       </c>
       <c r="C255" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D255" s="5" t="inlineStr">
         <is>
@@ -6865,7 +6865,7 @@
     <row r="256">
       <c r="A256" s="6" t="inlineStr">
         <is>
-          <t>Riyadh Marathon (Half)</t>
+          <t>NYCRUNS Brooklyn Experience Half Marathon</t>
         </is>
       </c>
       <c r="B256" s="7" t="inlineStr">
@@ -6874,7 +6874,7 @@
         </is>
       </c>
       <c r="C256" s="7" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D256" s="7" t="inlineStr">
         <is>
@@ -6890,7 +6890,7 @@
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>Riyadh Marathon (Half)</t>
+          <t>NYRR RBC Brooklyn Half</t>
         </is>
       </c>
       <c r="B257" s="5" t="inlineStr">
@@ -6899,7 +6899,7 @@
         </is>
       </c>
       <c r="C257" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D257" s="5" t="inlineStr">
         <is>
@@ -6915,7 +6915,7 @@
     <row r="258">
       <c r="A258" s="6" t="inlineStr">
         <is>
-          <t>Riyadh Marathon (Half)</t>
+          <t>Nike Melbourne Marathon Festival</t>
         </is>
       </c>
       <c r="B258" s="7" t="inlineStr">
@@ -6949,7 +6949,7 @@
         </is>
       </c>
       <c r="C259" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D259" s="5" t="inlineStr">
         <is>
@@ -6965,7 +6965,7 @@
     <row r="260">
       <c r="A260" s="6" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Las Vegas</t>
+          <t>Riyadh Marathon (Half)</t>
         </is>
       </c>
       <c r="B260" s="7" t="inlineStr">
@@ -6974,7 +6974,7 @@
         </is>
       </c>
       <c r="C260" s="7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D260" s="7" t="inlineStr">
         <is>
@@ -6990,7 +6990,7 @@
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Las Vegas</t>
+          <t>Riyadh Marathon (Half)</t>
         </is>
       </c>
       <c r="B261" s="5" t="inlineStr">
@@ -6999,7 +6999,7 @@
         </is>
       </c>
       <c r="C261" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D261" s="5" t="inlineStr">
         <is>
@@ -7015,7 +7015,7 @@
     <row r="262">
       <c r="A262" s="6" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Las Vegas</t>
+          <t>Riyadh Marathon (Half)</t>
         </is>
       </c>
       <c r="B262" s="7" t="inlineStr">
@@ -7024,7 +7024,7 @@
         </is>
       </c>
       <c r="C262" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D262" s="7" t="inlineStr">
         <is>
@@ -7049,7 +7049,7 @@
         </is>
       </c>
       <c r="C263" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D263" s="5" t="inlineStr">
         <is>
@@ -7065,7 +7065,7 @@
     <row r="264">
       <c r="A264" s="6" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Mexico City</t>
+          <t>Rock 'n' Roll Running Series Las Vegas</t>
         </is>
       </c>
       <c r="B264" s="7" t="inlineStr">
@@ -7074,7 +7074,7 @@
         </is>
       </c>
       <c r="C264" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D264" s="7" t="inlineStr">
         <is>
@@ -7090,7 +7090,7 @@
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series San Diego</t>
+          <t>Rock 'n' Roll Running Series Las Vegas</t>
         </is>
       </c>
       <c r="B265" s="5" t="inlineStr">
@@ -7115,7 +7115,7 @@
     <row r="266">
       <c r="A266" s="6" t="inlineStr">
         <is>
-          <t>Royal Parks Half Marathon</t>
+          <t>Rock 'n' Roll Running Series Las Vegas</t>
         </is>
       </c>
       <c r="B266" s="7" t="inlineStr">
@@ -7124,7 +7124,7 @@
         </is>
       </c>
       <c r="C266" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D266" s="7" t="inlineStr">
         <is>
@@ -7140,7 +7140,7 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (Semi)</t>
+          <t>Rock 'n' Roll Running Series Mexico City</t>
         </is>
       </c>
       <c r="B267" s="5" t="inlineStr">
@@ -7149,7 +7149,7 @@
         </is>
       </c>
       <c r="C267" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D267" s="5" t="inlineStr">
         <is>
@@ -7165,7 +7165,7 @@
     <row r="268">
       <c r="A268" s="6" t="inlineStr">
         <is>
-          <t>Run in Lyon (Semi)</t>
+          <t>Rock 'n' Roll Running Series San Diego</t>
         </is>
       </c>
       <c r="B268" s="7" t="inlineStr">
@@ -7174,23 +7174,23 @@
         </is>
       </c>
       <c r="C268" s="7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D268" s="7" t="inlineStr">
         <is>
-          <t>1:05:44</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E268" s="7" t="inlineStr">
         <is>
-          <t>1:18:34</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (Semi)</t>
+          <t>Royal Parks Half Marathon</t>
         </is>
       </c>
       <c r="B269" s="5" t="inlineStr">
@@ -7215,7 +7215,7 @@
     <row r="270">
       <c r="A270" s="6" t="inlineStr">
         <is>
-          <t>Semi-Marathon de Boulogne-Billancourt</t>
+          <t>Run in Lyon (Semi)</t>
         </is>
       </c>
       <c r="B270" s="7" t="inlineStr">
@@ -7224,7 +7224,7 @@
         </is>
       </c>
       <c r="C270" s="7" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D270" s="7" t="inlineStr">
         <is>
@@ -7240,7 +7240,7 @@
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>St. Jude Rock 'n' Roll Running Series Washington DC</t>
+          <t>Run in Lyon (Semi)</t>
         </is>
       </c>
       <c r="B271" s="5" t="inlineStr">
@@ -7249,23 +7249,23 @@
         </is>
       </c>
       <c r="C271" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D271" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:05:44</t>
         </is>
       </c>
       <c r="E271" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:18:34</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="6" t="inlineStr">
         <is>
-          <t>St. Jude Rock 'n' Roll Series Nashville</t>
+          <t>Run in Lyon (Semi)</t>
         </is>
       </c>
       <c r="B272" s="7" t="inlineStr">
@@ -7290,7 +7290,7 @@
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered Hong Kong Half Marathon</t>
+          <t>Semi-Marathon de Boulogne-Billancourt</t>
         </is>
       </c>
       <c r="B273" s="5" t="inlineStr">
@@ -7315,7 +7315,7 @@
     <row r="274">
       <c r="A274" s="6" t="inlineStr">
         <is>
-          <t>Standard Chartered Singapore Half Marathon</t>
+          <t>St. Jude Rock 'n' Roll Running Series Washington DC</t>
         </is>
       </c>
       <c r="B274" s="7" t="inlineStr">
@@ -7340,7 +7340,7 @@
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>TCS Mizuno Half Marathon</t>
+          <t>St. Jude Rock 'n' Roll Series Nashville</t>
         </is>
       </c>
       <c r="B275" s="5" t="inlineStr">
@@ -7365,7 +7365,7 @@
     <row r="276">
       <c r="A276" s="6" t="inlineStr">
         <is>
-          <t>TCS Toronto Waterfront Marathon (Half)</t>
+          <t>Standard Chartered Hong Kong Half Marathon</t>
         </is>
       </c>
       <c r="B276" s="7" t="inlineStr">
@@ -7374,7 +7374,7 @@
         </is>
       </c>
       <c r="C276" s="7" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D276" s="7" t="inlineStr">
         <is>
@@ -7390,7 +7390,7 @@
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>TCS Toronto Waterfront Marathon (Half)</t>
+          <t>Standard Chartered Singapore Half Marathon</t>
         </is>
       </c>
       <c r="B277" s="5" t="inlineStr">
@@ -7399,7 +7399,7 @@
         </is>
       </c>
       <c r="C277" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D277" s="5" t="inlineStr">
         <is>
@@ -7415,7 +7415,7 @@
     <row r="278">
       <c r="A278" s="6" t="inlineStr">
         <is>
-          <t>TCS Toronto Waterfront Marathon (Half)</t>
+          <t>TCS Mizuno Half Marathon</t>
         </is>
       </c>
       <c r="B278" s="7" t="inlineStr">
@@ -7440,7 +7440,7 @@
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>Taipei Half Marathon</t>
+          <t>TCS Toronto Waterfront Marathon (Half)</t>
         </is>
       </c>
       <c r="B279" s="5" t="inlineStr">
@@ -7465,7 +7465,7 @@
     <row r="280">
       <c r="A280" s="6" t="inlineStr">
         <is>
-          <t>Taipei Half Marathon</t>
+          <t>TCS Toronto Waterfront Marathon (Half)</t>
         </is>
       </c>
       <c r="B280" s="7" t="inlineStr">
@@ -7490,7 +7490,7 @@
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
         <is>
-          <t>Taipei Half Marathon</t>
+          <t>TCS Toronto Waterfront Marathon (Half)</t>
         </is>
       </c>
       <c r="B281" s="5" t="inlineStr">
@@ -7515,7 +7515,7 @@
     <row r="282">
       <c r="A282" s="6" t="inlineStr">
         <is>
-          <t>Tata Mumbai Marathon (Half)</t>
+          <t>Taipei Half Marathon</t>
         </is>
       </c>
       <c r="B282" s="7" t="inlineStr">
@@ -7524,7 +7524,7 @@
         </is>
       </c>
       <c r="C282" s="7" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D282" s="7" t="inlineStr">
         <is>
@@ -7540,7 +7540,7 @@
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>Tata Mumbai Marathon (Half)</t>
+          <t>Taipei Half Marathon</t>
         </is>
       </c>
       <c r="B283" s="5" t="inlineStr">
@@ -7549,7 +7549,7 @@
         </is>
       </c>
       <c r="C283" s="5" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D283" s="5" t="inlineStr">
         <is>
@@ -7565,7 +7565,7 @@
     <row r="284">
       <c r="A284" s="6" t="inlineStr">
         <is>
-          <t>The Big Half</t>
+          <t>Taipei Half Marathon</t>
         </is>
       </c>
       <c r="B284" s="7" t="inlineStr">
@@ -7590,7 +7590,7 @@
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>Tokyo Legacy Half Marathon</t>
+          <t>Tata Mumbai Marathon (Half)</t>
         </is>
       </c>
       <c r="B285" s="5" t="inlineStr">
@@ -7615,7 +7615,7 @@
     <row r="286">
       <c r="A286" s="6" t="inlineStr">
         <is>
-          <t>United Airlines NYC Half</t>
+          <t>Tata Mumbai Marathon (Half)</t>
         </is>
       </c>
       <c r="B286" s="7" t="inlineStr">
@@ -7624,23 +7624,23 @@
         </is>
       </c>
       <c r="C286" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D286" s="7" t="inlineStr">
         <is>
-          <t>1:01:31</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E286" s="7" t="inlineStr">
         <is>
-          <t>1:07:04</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>United Airlines NYC Half</t>
+          <t>The Big Half</t>
         </is>
       </c>
       <c r="B287" s="5" t="inlineStr">
@@ -7649,23 +7649,23 @@
         </is>
       </c>
       <c r="C287" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D287" s="5" t="inlineStr">
         <is>
-          <t>0:59:30</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E287" s="5" t="inlineStr">
         <is>
-          <t>1:06:33</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="6" t="inlineStr">
         <is>
-          <t>Valencia Half Marathon Trinidad Alfonso Zurich</t>
+          <t>Tokyo Legacy Half Marathon</t>
         </is>
       </c>
       <c r="B288" s="7" t="inlineStr">
@@ -7678,19 +7678,19 @@
       </c>
       <c r="D288" s="7" t="inlineStr">
         <is>
-          <t>0:58:02</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E288" s="7" t="inlineStr">
         <is>
-          <t>1:03:08</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>Vedanta Delhi Half Marathon</t>
+          <t>United Airlines NYC Half</t>
         </is>
       </c>
       <c r="B289" s="5" t="inlineStr">
@@ -7703,19 +7703,19 @@
       </c>
       <c r="D289" s="5" t="inlineStr">
         <is>
-          <t>0:59:50</t>
+          <t>1:01:31</t>
         </is>
       </c>
       <c r="E289" s="5" t="inlineStr">
         <is>
-          <t>1:07:20</t>
+          <t>1:07:04</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="6" t="inlineStr">
         <is>
-          <t>Vienna City Half Marathon</t>
+          <t>United Airlines NYC Half</t>
         </is>
       </c>
       <c r="B290" s="7" t="inlineStr">
@@ -7724,23 +7724,23 @@
         </is>
       </c>
       <c r="C290" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D290" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:30</t>
         </is>
       </c>
       <c r="E290" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:33</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>Walt Disney World Marathon Weekend</t>
+          <t>Valencia Half Marathon Trinidad Alfonso Zurich</t>
         </is>
       </c>
       <c r="B291" s="5" t="inlineStr">
@@ -7753,19 +7753,19 @@
       </c>
       <c r="D291" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:58:02</t>
         </is>
       </c>
       <c r="E291" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:03:08</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="6" t="inlineStr">
         <is>
-          <t>Walt Disney World Marathon Weekend</t>
+          <t>Vedanta Delhi Half Marathon</t>
         </is>
       </c>
       <c r="B292" s="7" t="inlineStr">
@@ -7774,23 +7774,23 @@
         </is>
       </c>
       <c r="C292" s="7" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D292" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:50</t>
         </is>
       </c>
       <c r="E292" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:07:20</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>Warsaw Half Marathon</t>
+          <t>Vienna City Half Marathon</t>
         </is>
       </c>
       <c r="B293" s="5" t="inlineStr">
@@ -7799,7 +7799,7 @@
         </is>
       </c>
       <c r="C293" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D293" s="5" t="inlineStr">
         <is>
@@ -7815,7 +7815,7 @@
     <row r="294">
       <c r="A294" s="6" t="inlineStr">
         <is>
-          <t>Warsaw Half Marathon</t>
+          <t>Walt Disney World Marathon Weekend</t>
         </is>
       </c>
       <c r="B294" s="7" t="inlineStr">
@@ -7840,7 +7840,7 @@
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>Wizz Air Rome Half Marathon by Brooks</t>
+          <t>Walt Disney World Marathon Weekend</t>
         </is>
       </c>
       <c r="B295" s="5" t="inlineStr">
@@ -7849,7 +7849,7 @@
         </is>
       </c>
       <c r="C295" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D295" s="5" t="inlineStr">
         <is>
@@ -7865,7 +7865,7 @@
     <row r="296">
       <c r="A296" s="6" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+          <t>Warsaw Half Marathon</t>
         </is>
       </c>
       <c r="B296" s="7" t="inlineStr">
@@ -7874,7 +7874,7 @@
         </is>
       </c>
       <c r="C296" s="7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D296" s="7" t="inlineStr">
         <is>
@@ -7890,7 +7890,7 @@
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+          <t>Warsaw Half Marathon</t>
         </is>
       </c>
       <c r="B297" s="5" t="inlineStr">
@@ -7899,7 +7899,7 @@
         </is>
       </c>
       <c r="C297" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D297" s="5" t="inlineStr">
         <is>
@@ -7915,7 +7915,7 @@
     <row r="298">
       <c r="A298" s="6" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+          <t>Wizz Air Rome Half Marathon by Brooks</t>
         </is>
       </c>
       <c r="B298" s="7" t="inlineStr">
@@ -7940,16 +7940,16 @@
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>10K Montmartre</t>
+          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
         </is>
       </c>
       <c r="B299" s="5" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>21K</t>
         </is>
       </c>
       <c r="C299" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D299" s="5" t="inlineStr">
         <is>
@@ -7963,43 +7963,43 @@
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="8" t="inlineStr">
-        <is>
-          <t>10K Valencia Ibercaja by Kiprun</t>
-        </is>
-      </c>
-      <c r="B300" s="9" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
-      <c r="C300" s="9" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D300" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E300" s="9" t="inlineStr">
-        <is>
-          <t>0:29:19</t>
+      <c r="A300" s="6" t="inlineStr">
+        <is>
+          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+        </is>
+      </c>
+      <c r="B300" s="7" t="inlineStr">
+        <is>
+          <t>21K</t>
+        </is>
+      </c>
+      <c r="C300" s="7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D300" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E300" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>10K Valencia Ibercaja by Kiprun</t>
+          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
         </is>
       </c>
       <c r="B301" s="5" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>21K</t>
         </is>
       </c>
       <c r="C301" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D301" s="5" t="inlineStr">
         <is>
@@ -8008,14 +8008,14 @@
       </c>
       <c r="E301" s="5" t="inlineStr">
         <is>
-          <t>0:28:45</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="8" t="inlineStr">
         <is>
-          <t>10K Valencia Ibercaja by Kiprun</t>
+          <t>10K Montmartre</t>
         </is>
       </c>
       <c r="B302" s="9" t="inlineStr">
@@ -8024,7 +8024,7 @@
         </is>
       </c>
       <c r="C302" s="9" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D302" s="9" t="inlineStr">
         <is>
@@ -8049,23 +8049,23 @@
         </is>
       </c>
       <c r="C303" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D303" s="5" t="inlineStr">
         <is>
-          <t>0:26:45</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E303" s="5" t="inlineStr">
         <is>
-          <t>0:29:25</t>
+          <t>0:29:19</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run (10K)</t>
+          <t>10K Valencia Ibercaja by Kiprun</t>
         </is>
       </c>
       <c r="B304" s="9" t="inlineStr">
@@ -8083,14 +8083,14 @@
       </c>
       <c r="E304" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:45</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run (10K)</t>
+          <t>10K Valencia Ibercaja by Kiprun</t>
         </is>
       </c>
       <c r="B305" s="5" t="inlineStr">
@@ -8115,7 +8115,7 @@
     <row r="306">
       <c r="A306" s="8" t="inlineStr">
         <is>
-          <t>ASICS LDNX</t>
+          <t>10K Valencia Ibercaja by Kiprun</t>
         </is>
       </c>
       <c r="B306" s="9" t="inlineStr">
@@ -8124,23 +8124,23 @@
         </is>
       </c>
       <c r="C306" s="9" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D306" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:26:45</t>
         </is>
       </c>
       <c r="E306" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:25</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>AJ Bell Great Manchester Run (10K)</t>
         </is>
       </c>
       <c r="B307" s="5" t="inlineStr">
@@ -8149,7 +8149,7 @@
         </is>
       </c>
       <c r="C307" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D307" s="5" t="inlineStr">
         <is>
@@ -8165,7 +8165,7 @@
     <row r="308">
       <c r="A308" s="8" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>AJ Bell Great Manchester Run (10K)</t>
         </is>
       </c>
       <c r="B308" s="9" t="inlineStr">
@@ -8174,23 +8174,23 @@
         </is>
       </c>
       <c r="C308" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D308" s="9" t="inlineStr">
         <is>
-          <t>0:29:37</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E308" s="9" t="inlineStr">
         <is>
-          <t>0:32:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>ASICS LDNX</t>
         </is>
       </c>
       <c r="B309" s="5" t="inlineStr">
@@ -8215,7 +8215,7 @@
     <row r="310">
       <c r="A310" s="8" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B310" s="9" t="inlineStr">
@@ -8228,19 +8228,19 @@
       </c>
       <c r="D310" s="9" t="inlineStr">
         <is>
-          <t>0:27:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E310" s="9" t="inlineStr">
         <is>
-          <t>0:30:43</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B311" s="5" t="inlineStr">
@@ -8253,19 +8253,19 @@
       </c>
       <c r="D311" s="5" t="inlineStr">
         <is>
-          <t>0:28:03</t>
+          <t>0:29:37</t>
         </is>
       </c>
       <c r="E311" s="5" t="inlineStr">
         <is>
-          <t>0:31:12</t>
+          <t>0:32:18</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="8" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B312" s="9" t="inlineStr">
@@ -8283,14 +8283,14 @@
       </c>
       <c r="E312" s="9" t="inlineStr">
         <is>
-          <t>0:31:29</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B313" s="5" t="inlineStr">
@@ -8303,19 +8303,19 @@
       </c>
       <c r="D313" s="5" t="inlineStr">
         <is>
-          <t>0:29:08</t>
+          <t>0:27:41</t>
         </is>
       </c>
       <c r="E313" s="5" t="inlineStr">
         <is>
-          <t>0:33:25</t>
+          <t>0:30:43</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="8" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B314" s="9" t="inlineStr">
@@ -8328,19 +8328,19 @@
       </c>
       <c r="D314" s="9" t="inlineStr">
         <is>
-          <t>0:29:13</t>
+          <t>0:28:03</t>
         </is>
       </c>
       <c r="E314" s="9" t="inlineStr">
         <is>
-          <t>0:32:45</t>
+          <t>0:31:12</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B315" s="5" t="inlineStr">
@@ -8358,14 +8358,14 @@
       </c>
       <c r="E315" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:29</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="8" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B316" s="9" t="inlineStr">
@@ -8378,19 +8378,19 @@
       </c>
       <c r="D316" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:08</t>
         </is>
       </c>
       <c r="E316" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:33:25</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B317" s="5" t="inlineStr">
@@ -8403,19 +8403,19 @@
       </c>
       <c r="D317" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:13</t>
         </is>
       </c>
       <c r="E317" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:45</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="8" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B318" s="9" t="inlineStr">
@@ -8440,7 +8440,7 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B319" s="5" t="inlineStr">
@@ -8453,19 +8453,19 @@
       </c>
       <c r="D319" s="5" t="inlineStr">
         <is>
-          <t>0:28:52</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E319" s="5" t="inlineStr">
         <is>
-          <t>0:31:59</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="8" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B320" s="9" t="inlineStr">
@@ -8478,19 +8478,19 @@
       </c>
       <c r="D320" s="9" t="inlineStr">
         <is>
-          <t>0:28:46</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E320" s="9" t="inlineStr">
         <is>
-          <t>0:32:33</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B321" s="5" t="inlineStr">
@@ -8503,12 +8503,12 @@
       </c>
       <c r="D321" s="5" t="inlineStr">
         <is>
-          <t>0:29:22</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E321" s="5" t="inlineStr">
         <is>
-          <t>0:34:32</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -8524,23 +8524,23 @@
         </is>
       </c>
       <c r="C322" s="9" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D322" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:52</t>
         </is>
       </c>
       <c r="E322" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:59</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B323" s="5" t="inlineStr">
@@ -8549,23 +8549,23 @@
         </is>
       </c>
       <c r="C323" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D323" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:46</t>
         </is>
       </c>
       <c r="E323" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:33</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="8" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B324" s="9" t="inlineStr">
@@ -8574,23 +8574,23 @@
         </is>
       </c>
       <c r="C324" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D324" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:22</t>
         </is>
       </c>
       <c r="E324" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:34:32</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B325" s="5" t="inlineStr">
@@ -8599,23 +8599,23 @@
         </is>
       </c>
       <c r="C325" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D325" s="5" t="inlineStr">
         <is>
-          <t>0:28:27</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E325" s="5" t="inlineStr">
         <is>
-          <t>0:31:49</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="8" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B326" s="9" t="inlineStr">
@@ -8640,7 +8640,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B327" s="5" t="inlineStr">
@@ -8665,7 +8665,7 @@
     <row r="328">
       <c r="A328" s="8" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B328" s="9" t="inlineStr">
@@ -8678,12 +8678,12 @@
       </c>
       <c r="D328" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:27</t>
         </is>
       </c>
       <c r="E328" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:49</t>
         </is>
       </c>
     </row>
@@ -8699,7 +8699,7 @@
         </is>
       </c>
       <c r="C329" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D329" s="5" t="inlineStr">
         <is>
@@ -8715,7 +8715,7 @@
     <row r="330">
       <c r="A330" s="8" t="inlineStr">
         <is>
-          <t>NN CPC Loop Den Haag - 10 KM Loop</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B330" s="9" t="inlineStr">
@@ -8724,7 +8724,7 @@
         </is>
       </c>
       <c r="C330" s="9" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D330" s="9" t="inlineStr">
         <is>
@@ -8740,7 +8740,7 @@
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B331" s="5" t="inlineStr">
@@ -8749,7 +8749,7 @@
         </is>
       </c>
       <c r="C331" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D331" s="5" t="inlineStr">
         <is>
@@ -8765,7 +8765,7 @@
     <row r="332">
       <c r="A332" s="8" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B332" s="9" t="inlineStr">
@@ -8774,7 +8774,7 @@
         </is>
       </c>
       <c r="C332" s="9" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D332" s="9" t="inlineStr">
         <is>
@@ -8783,14 +8783,14 @@
       </c>
       <c r="E332" s="9" t="inlineStr">
         <is>
-          <t>0:31:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>NN CPC Loop Den Haag - 10 KM Loop</t>
         </is>
       </c>
       <c r="B333" s="5" t="inlineStr">
@@ -8799,23 +8799,23 @@
         </is>
       </c>
       <c r="C333" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D333" s="5" t="inlineStr">
         <is>
-          <t>0:27:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E333" s="5" t="inlineStr">
         <is>
-          <t>0:31:11</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="8" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B334" s="9" t="inlineStr">
@@ -8840,7 +8840,7 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B335" s="5" t="inlineStr">
@@ -8858,14 +8858,14 @@
       </c>
       <c r="E335" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:18</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="8" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B336" s="9" t="inlineStr">
@@ -8878,19 +8878,19 @@
       </c>
       <c r="D336" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:27:41</t>
         </is>
       </c>
       <c r="E336" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:11</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B337" s="5" t="inlineStr">
@@ -8915,7 +8915,7 @@
     <row r="338">
       <c r="A338" s="8" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B338" s="9" t="inlineStr">
@@ -8940,7 +8940,7 @@
     <row r="339">
       <c r="A339" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B339" s="5" t="inlineStr">
@@ -8965,7 +8965,7 @@
     <row r="340">
       <c r="A340" s="8" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B340" s="9" t="inlineStr">
@@ -8990,7 +8990,7 @@
     <row r="341">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B341" s="5" t="inlineStr">
@@ -9003,19 +9003,19 @@
       </c>
       <c r="D341" s="5" t="inlineStr">
         <is>
-          <t>0:29:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E341" s="5" t="inlineStr">
         <is>
-          <t>0:32:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="8" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B342" s="9" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="D342" s="9" t="inlineStr">
         <is>
-          <t>0:29:33</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E342" s="9" t="inlineStr">
@@ -9040,7 +9040,7 @@
     <row r="343">
       <c r="A343" s="4" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B343" s="5" t="inlineStr">
@@ -9065,7 +9065,7 @@
     <row r="344">
       <c r="A344" s="8" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B344" s="9" t="inlineStr">
@@ -9078,19 +9078,19 @@
       </c>
       <c r="D344" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:41</t>
         </is>
       </c>
       <c r="E344" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:51</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B345" s="5" t="inlineStr">
@@ -9103,7 +9103,7 @@
       </c>
       <c r="D345" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:33</t>
         </is>
       </c>
       <c r="E345" s="5" t="inlineStr">
@@ -9115,7 +9115,7 @@
     <row r="346">
       <c r="A346" s="8" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B346" s="9" t="inlineStr">
@@ -9140,7 +9140,7 @@
     <row r="347">
       <c r="A347" s="4" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B347" s="5" t="inlineStr">
@@ -9165,7 +9165,7 @@
     <row r="348">
       <c r="A348" s="8" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B348" s="9" t="inlineStr">
@@ -9190,7 +9190,7 @@
     <row r="349">
       <c r="A349" s="4" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B349" s="5" t="inlineStr">
@@ -9215,7 +9215,7 @@
     <row r="350">
       <c r="A350" s="8" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B350" s="9" t="inlineStr">
@@ -9240,7 +9240,7 @@
     <row r="351">
       <c r="A351" s="4" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B351" s="5" t="inlineStr">
@@ -9265,7 +9265,7 @@
     <row r="352">
       <c r="A352" s="8" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Ukrop's Monument Avenue 10K</t>
         </is>
       </c>
       <c r="B352" s="9" t="inlineStr">
@@ -9290,7 +9290,7 @@
     <row r="353">
       <c r="A353" s="4" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Ukrop's Monument Avenue 10K</t>
         </is>
       </c>
       <c r="B353" s="5" t="inlineStr">
@@ -9315,7 +9315,7 @@
     <row r="354">
       <c r="A354" s="8" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Ukrop's Monument Avenue 10K</t>
         </is>
       </c>
       <c r="B354" s="9" t="inlineStr">
@@ -9328,19 +9328,19 @@
       </c>
       <c r="D354" s="9" t="inlineStr">
         <is>
-          <t>0:28:09</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E354" s="9" t="inlineStr">
         <is>
-          <t>0:32:54</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="4" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Vancouver Sun Run</t>
         </is>
       </c>
       <c r="B355" s="5" t="inlineStr">
@@ -9365,7 +9365,7 @@
     <row r="356">
       <c r="A356" s="8" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Vancouver Sun Run</t>
         </is>
       </c>
       <c r="B356" s="9" t="inlineStr">
@@ -9378,42 +9378,117 @@
       </c>
       <c r="D356" s="9" t="inlineStr">
         <is>
-          <t>0:29:14</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E356" s="9" t="inlineStr">
         <is>
-          <t>0:31:36</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="4" t="inlineStr">
         <is>
+          <t>Vancouver Sun Run</t>
+        </is>
+      </c>
+      <c r="B357" s="5" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C357" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D357" s="5" t="inlineStr">
+        <is>
+          <t>0:28:09</t>
+        </is>
+      </c>
+      <c r="E357" s="5" t="inlineStr">
+        <is>
+          <t>0:32:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="8" t="inlineStr">
+        <is>
           <t>Vitality London 10,000</t>
         </is>
       </c>
-      <c r="B357" s="5" t="inlineStr">
+      <c r="B358" s="9" t="inlineStr">
         <is>
           <t>10K</t>
         </is>
       </c>
-      <c r="C357" s="5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D357" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E357" s="5" t="inlineStr">
+      <c r="C358" s="9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D358" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E358" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="4" t="inlineStr">
+        <is>
+          <t>Vitality London 10,000</t>
+        </is>
+      </c>
+      <c r="B359" s="5" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C359" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D359" s="5" t="inlineStr">
+        <is>
+          <t>0:29:14</t>
+        </is>
+      </c>
+      <c r="E359" s="5" t="inlineStr">
+        <is>
+          <t>0:31:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="8" t="inlineStr">
+        <is>
+          <t>Vitality London 10,000</t>
+        </is>
+      </c>
+      <c r="B360" s="9" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C360" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D360" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E360" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E357"/>
+  <autoFilter ref="A1:E360"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 25+ winner times: AUTRE events, 10K, HM + AUTRE filter in Winners tab
Added winner times for:
- Dam tot Damloop 2019/2024/2025
- Bay to Breakers 2019/2022/2024
- Broad Street Run, Boilermaker, BOLDERBoulder 2025
- KLSCM (marathon+half+10K) 2025
- HK Marathon 2019
- 10+ other 10K/SEMI/AUTRE events
Added "Autre" distance filter in Winners Times tab.
Total: 137 unique courses, 390 result lines.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$366</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$391</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E366"/>
+  <dimension ref="A1:E391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -8290,7 +8290,7 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run (10K)</t>
+          <t>AJ Bell Great Birmingham Run 10K</t>
         </is>
       </c>
       <c r="B313" s="5" t="inlineStr">
@@ -8299,7 +8299,7 @@
         </is>
       </c>
       <c r="C313" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D313" s="5" t="inlineStr">
         <is>
@@ -8315,7 +8315,7 @@
     <row r="314">
       <c r="A314" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run (10K)</t>
+          <t>AJ Bell Great Bristol Run 10K</t>
         </is>
       </c>
       <c r="B314" s="9" t="inlineStr">
@@ -8340,7 +8340,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>ASICS LDNX</t>
+          <t>AJ Bell Great Manchester Run</t>
         </is>
       </c>
       <c r="B315" s="5" t="inlineStr">
@@ -8365,7 +8365,7 @@
     <row r="316">
       <c r="A316" s="8" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>AJ Bell Great Manchester Run (10K)</t>
         </is>
       </c>
       <c r="B316" s="9" t="inlineStr">
@@ -8374,7 +8374,7 @@
         </is>
       </c>
       <c r="C316" s="9" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D316" s="9" t="inlineStr">
         <is>
@@ -8390,7 +8390,7 @@
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>AJ Bell Great Manchester Run (10K)</t>
         </is>
       </c>
       <c r="B317" s="5" t="inlineStr">
@@ -8399,23 +8399,23 @@
         </is>
       </c>
       <c r="C317" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D317" s="5" t="inlineStr">
         <is>
-          <t>0:29:37</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E317" s="5" t="inlineStr">
         <is>
-          <t>0:32:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="8" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>AJ Bell Great North 10K</t>
         </is>
       </c>
       <c r="B318" s="9" t="inlineStr">
@@ -8440,7 +8440,7 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>ASICS LDNX</t>
         </is>
       </c>
       <c r="B319" s="5" t="inlineStr">
@@ -8449,23 +8449,23 @@
         </is>
       </c>
       <c r="C319" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D319" s="5" t="inlineStr">
         <is>
-          <t>0:27:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E319" s="5" t="inlineStr">
         <is>
-          <t>0:30:43</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="8" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B320" s="9" t="inlineStr">
@@ -8474,23 +8474,23 @@
         </is>
       </c>
       <c r="C320" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D320" s="9" t="inlineStr">
         <is>
-          <t>0:28:03</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E320" s="9" t="inlineStr">
         <is>
-          <t>0:31:12</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B321" s="5" t="inlineStr">
@@ -8499,23 +8499,23 @@
         </is>
       </c>
       <c r="C321" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D321" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:37</t>
         </is>
       </c>
       <c r="E321" s="5" t="inlineStr">
         <is>
-          <t>0:31:29</t>
+          <t>0:32:18</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="8" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B322" s="9" t="inlineStr">
@@ -8524,23 +8524,23 @@
         </is>
       </c>
       <c r="C322" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D322" s="9" t="inlineStr">
         <is>
-          <t>0:29:08</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E322" s="9" t="inlineStr">
         <is>
-          <t>0:33:25</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B323" s="5" t="inlineStr">
@@ -8549,23 +8549,23 @@
         </is>
       </c>
       <c r="C323" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D323" s="5" t="inlineStr">
         <is>
-          <t>0:29:13</t>
+          <t>0:27:41</t>
         </is>
       </c>
       <c r="E323" s="5" t="inlineStr">
         <is>
-          <t>0:32:45</t>
+          <t>0:30:43</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="8" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B324" s="9" t="inlineStr">
@@ -8574,23 +8574,23 @@
         </is>
       </c>
       <c r="C324" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D324" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:03</t>
         </is>
       </c>
       <c r="E324" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:12</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B325" s="5" t="inlineStr">
@@ -8599,7 +8599,7 @@
         </is>
       </c>
       <c r="C325" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D325" s="5" t="inlineStr">
         <is>
@@ -8608,14 +8608,14 @@
       </c>
       <c r="E325" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:29</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="8" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B326" s="9" t="inlineStr">
@@ -8624,23 +8624,23 @@
         </is>
       </c>
       <c r="C326" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D326" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:08</t>
         </is>
       </c>
       <c r="E326" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:33:25</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B327" s="5" t="inlineStr">
@@ -8649,23 +8649,23 @@
         </is>
       </c>
       <c r="C327" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D327" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:13</t>
         </is>
       </c>
       <c r="E327" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:45</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="8" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B328" s="9" t="inlineStr">
@@ -8674,23 +8674,23 @@
         </is>
       </c>
       <c r="C328" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D328" s="9" t="inlineStr">
         <is>
-          <t>0:28:52</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E328" s="9" t="inlineStr">
         <is>
-          <t>0:31:59</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B329" s="5" t="inlineStr">
@@ -8699,23 +8699,23 @@
         </is>
       </c>
       <c r="C329" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D329" s="5" t="inlineStr">
         <is>
-          <t>0:28:46</t>
+          <t>0:28:36</t>
         </is>
       </c>
       <c r="E329" s="5" t="inlineStr">
         <is>
-          <t>0:32:33</t>
+          <t>0:31:51</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="8" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B330" s="9" t="inlineStr">
@@ -8724,23 +8724,23 @@
         </is>
       </c>
       <c r="C330" s="9" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D330" s="9" t="inlineStr">
         <is>
-          <t>0:29:22</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E330" s="9" t="inlineStr">
         <is>
-          <t>0:34:32</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B331" s="5" t="inlineStr">
@@ -8749,7 +8749,7 @@
         </is>
       </c>
       <c r="C331" s="5" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D331" s="5" t="inlineStr">
         <is>
@@ -8765,7 +8765,7 @@
     <row r="332">
       <c r="A332" s="8" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B332" s="9" t="inlineStr">
@@ -8774,7 +8774,7 @@
         </is>
       </c>
       <c r="C332" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D332" s="9" t="inlineStr">
         <is>
@@ -8790,7 +8790,7 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B333" s="5" t="inlineStr">
@@ -8799,23 +8799,23 @@
         </is>
       </c>
       <c r="C333" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D333" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:52</t>
         </is>
       </c>
       <c r="E333" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:59</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="8" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B334" s="9" t="inlineStr">
@@ -8824,23 +8824,23 @@
         </is>
       </c>
       <c r="C334" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D334" s="9" t="inlineStr">
         <is>
-          <t>0:28:27</t>
+          <t>0:28:46</t>
         </is>
       </c>
       <c r="E334" s="9" t="inlineStr">
         <is>
-          <t>0:31:49</t>
+          <t>0:32:33</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B335" s="5" t="inlineStr">
@@ -8849,23 +8849,23 @@
         </is>
       </c>
       <c r="C335" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D335" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:22</t>
         </is>
       </c>
       <c r="E335" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:34:32</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="8" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B336" s="9" t="inlineStr">
@@ -8874,7 +8874,7 @@
         </is>
       </c>
       <c r="C336" s="9" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D336" s="9" t="inlineStr">
         <is>
@@ -8890,7 +8890,7 @@
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B337" s="5" t="inlineStr">
@@ -8899,7 +8899,7 @@
         </is>
       </c>
       <c r="C337" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D337" s="5" t="inlineStr">
         <is>
@@ -8915,7 +8915,7 @@
     <row r="338">
       <c r="A338" s="8" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B338" s="9" t="inlineStr">
@@ -8924,7 +8924,7 @@
         </is>
       </c>
       <c r="C338" s="9" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D338" s="9" t="inlineStr">
         <is>
@@ -8940,7 +8940,7 @@
     <row r="339">
       <c r="A339" s="4" t="inlineStr">
         <is>
-          <t>NN CPC Loop Den Haag - 10 KM Loop</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B339" s="5" t="inlineStr">
@@ -8949,23 +8949,23 @@
         </is>
       </c>
       <c r="C339" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D339" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:27</t>
         </is>
       </c>
       <c r="E339" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:49</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="8" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B340" s="9" t="inlineStr">
@@ -8974,7 +8974,7 @@
         </is>
       </c>
       <c r="C340" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D340" s="9" t="inlineStr">
         <is>
@@ -8990,7 +8990,7 @@
     <row r="341">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B341" s="5" t="inlineStr">
@@ -8999,7 +8999,7 @@
         </is>
       </c>
       <c r="C341" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D341" s="5" t="inlineStr">
         <is>
@@ -9008,14 +9008,14 @@
       </c>
       <c r="E341" s="5" t="inlineStr">
         <is>
-          <t>0:31:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="8" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B342" s="9" t="inlineStr">
@@ -9024,23 +9024,23 @@
         </is>
       </c>
       <c r="C342" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D342" s="9" t="inlineStr">
         <is>
-          <t>0:27:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E342" s="9" t="inlineStr">
         <is>
-          <t>0:31:11</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="4" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B343" s="5" t="inlineStr">
@@ -9049,7 +9049,7 @@
         </is>
       </c>
       <c r="C343" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D343" s="5" t="inlineStr">
         <is>
@@ -9065,7 +9065,7 @@
     <row r="344">
       <c r="A344" s="8" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B344" s="9" t="inlineStr">
@@ -9074,7 +9074,7 @@
         </is>
       </c>
       <c r="C344" s="9" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D344" s="9" t="inlineStr">
         <is>
@@ -9090,7 +9090,7 @@
     <row r="345">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>Great Scottish Run 10K</t>
         </is>
       </c>
       <c r="B345" s="5" t="inlineStr">
@@ -9115,7 +9115,7 @@
     <row r="346">
       <c r="A346" s="8" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>NN CPC Loop Den Haag - 10 KM Loop</t>
         </is>
       </c>
       <c r="B346" s="9" t="inlineStr">
@@ -9124,7 +9124,7 @@
         </is>
       </c>
       <c r="C346" s="9" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D346" s="9" t="inlineStr">
         <is>
@@ -9140,7 +9140,7 @@
     <row r="347">
       <c r="A347" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B347" s="5" t="inlineStr">
@@ -9149,7 +9149,7 @@
         </is>
       </c>
       <c r="C347" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D347" s="5" t="inlineStr">
         <is>
@@ -9165,7 +9165,7 @@
     <row r="348">
       <c r="A348" s="8" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B348" s="9" t="inlineStr">
@@ -9174,7 +9174,7 @@
         </is>
       </c>
       <c r="C348" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D348" s="9" t="inlineStr">
         <is>
@@ -9183,14 +9183,14 @@
       </c>
       <c r="E348" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:18</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="4" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B349" s="5" t="inlineStr">
@@ -9199,23 +9199,23 @@
         </is>
       </c>
       <c r="C349" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D349" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:27:41</t>
         </is>
       </c>
       <c r="E349" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:11</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="8" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B350" s="9" t="inlineStr">
@@ -9224,23 +9224,23 @@
         </is>
       </c>
       <c r="C350" s="9" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D350" s="9" t="inlineStr">
         <is>
-          <t>0:29:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E350" s="9" t="inlineStr">
         <is>
-          <t>0:32:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="4" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B351" s="5" t="inlineStr">
@@ -9249,11 +9249,11 @@
         </is>
       </c>
       <c r="C351" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D351" s="5" t="inlineStr">
         <is>
-          <t>0:29:33</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E351" s="5" t="inlineStr">
@@ -9265,7 +9265,7 @@
     <row r="352">
       <c r="A352" s="8" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B352" s="9" t="inlineStr">
@@ -9274,7 +9274,7 @@
         </is>
       </c>
       <c r="C352" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D352" s="9" t="inlineStr">
         <is>
@@ -9290,7 +9290,7 @@
     <row r="353">
       <c r="A353" s="4" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Run in Lyon</t>
         </is>
       </c>
       <c r="B353" s="5" t="inlineStr">
@@ -9299,7 +9299,7 @@
         </is>
       </c>
       <c r="C353" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D353" s="5" t="inlineStr">
         <is>
@@ -9315,7 +9315,7 @@
     <row r="354">
       <c r="A354" s="8" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B354" s="9" t="inlineStr">
@@ -9324,7 +9324,7 @@
         </is>
       </c>
       <c r="C354" s="9" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D354" s="9" t="inlineStr">
         <is>
@@ -9340,7 +9340,7 @@
     <row r="355">
       <c r="A355" s="4" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B355" s="5" t="inlineStr">
@@ -9349,7 +9349,7 @@
         </is>
       </c>
       <c r="C355" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D355" s="5" t="inlineStr">
         <is>
@@ -9365,7 +9365,7 @@
     <row r="356">
       <c r="A356" s="8" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B356" s="9" t="inlineStr">
@@ -9374,7 +9374,7 @@
         </is>
       </c>
       <c r="C356" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D356" s="9" t="inlineStr">
         <is>
@@ -9390,7 +9390,7 @@
     <row r="357">
       <c r="A357" s="4" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B357" s="5" t="inlineStr">
@@ -9399,7 +9399,7 @@
         </is>
       </c>
       <c r="C357" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D357" s="5" t="inlineStr">
         <is>
@@ -9415,7 +9415,7 @@
     <row r="358">
       <c r="A358" s="8" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B358" s="9" t="inlineStr">
@@ -9424,23 +9424,23 @@
         </is>
       </c>
       <c r="C358" s="9" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D358" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:41</t>
         </is>
       </c>
       <c r="E358" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:51</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="4" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B359" s="5" t="inlineStr">
@@ -9449,11 +9449,11 @@
         </is>
       </c>
       <c r="C359" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D359" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:33</t>
         </is>
       </c>
       <c r="E359" s="5" t="inlineStr">
@@ -9465,7 +9465,7 @@
     <row r="360">
       <c r="A360" s="8" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Standard Chartered KL 10K</t>
         </is>
       </c>
       <c r="B360" s="9" t="inlineStr">
@@ -9478,19 +9478,19 @@
       </c>
       <c r="D360" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:26</t>
         </is>
       </c>
       <c r="E360" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:39:23</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="4" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B361" s="5" t="inlineStr">
@@ -9515,7 +9515,7 @@
     <row r="362">
       <c r="A362" s="8" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B362" s="9" t="inlineStr">
@@ -9540,7 +9540,7 @@
     <row r="363">
       <c r="A363" s="4" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B363" s="5" t="inlineStr">
@@ -9553,19 +9553,19 @@
       </c>
       <c r="D363" s="5" t="inlineStr">
         <is>
-          <t>0:28:09</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E363" s="5" t="inlineStr">
         <is>
-          <t>0:32:54</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="8" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B364" s="9" t="inlineStr">
@@ -9590,7 +9590,7 @@
     <row r="365">
       <c r="A365" s="4" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B365" s="5" t="inlineStr">
@@ -9603,42 +9603,667 @@
       </c>
       <c r="D365" s="5" t="inlineStr">
         <is>
-          <t>0:29:14</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E365" s="5" t="inlineStr">
         <is>
-          <t>0:31:36</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="8" t="inlineStr">
         <is>
+          <t>Transurban Bridge to Brisbane</t>
+        </is>
+      </c>
+      <c r="B366" s="9" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C366" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D366" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E366" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="4" t="inlineStr">
+        <is>
+          <t>Ukrop's Monument Avenue 10K</t>
+        </is>
+      </c>
+      <c r="B367" s="5" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C367" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D367" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E367" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="8" t="inlineStr">
+        <is>
+          <t>Ukrop's Monument Avenue 10K</t>
+        </is>
+      </c>
+      <c r="B368" s="9" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C368" s="9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D368" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E368" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="4" t="inlineStr">
+        <is>
+          <t>Ukrop's Monument Avenue 10K</t>
+        </is>
+      </c>
+      <c r="B369" s="5" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C369" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D369" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E369" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver Sun Run</t>
+        </is>
+      </c>
+      <c r="B370" s="9" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C370" s="9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D370" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E370" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver Sun Run</t>
+        </is>
+      </c>
+      <c r="B371" s="5" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C371" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D371" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E371" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="8" t="inlineStr">
+        <is>
+          <t>Vancouver Sun Run</t>
+        </is>
+      </c>
+      <c r="B372" s="9" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C372" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D372" s="9" t="inlineStr">
+        <is>
+          <t>0:28:09</t>
+        </is>
+      </c>
+      <c r="E372" s="9" t="inlineStr">
+        <is>
+          <t>0:32:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="4" t="inlineStr">
+        <is>
           <t>Vitality London 10,000</t>
         </is>
       </c>
-      <c r="B366" s="9" t="inlineStr">
+      <c r="B373" s="5" t="inlineStr">
         <is>
           <t>10K</t>
         </is>
       </c>
-      <c r="C366" s="9" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D366" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E366" s="9" t="inlineStr">
+      <c r="C373" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D373" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E373" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="8" t="inlineStr">
+        <is>
+          <t>Vitality London 10,000</t>
+        </is>
+      </c>
+      <c r="B374" s="9" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C374" s="9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D374" s="9" t="inlineStr">
+        <is>
+          <t>0:29:14</t>
+        </is>
+      </c>
+      <c r="E374" s="9" t="inlineStr">
+        <is>
+          <t>0:31:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="4" t="inlineStr">
+        <is>
+          <t>Vitality London 10,000</t>
+        </is>
+      </c>
+      <c r="B375" s="5" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="C375" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D375" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E375" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="8" t="inlineStr">
+        <is>
+          <t>AJ Bell Great Birmingham Run</t>
+        </is>
+      </c>
+      <c r="B376" s="9" t="inlineStr">
+        <is>
+          <t>SEMI</t>
+        </is>
+      </c>
+      <c r="C376" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D376" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E376" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="4" t="inlineStr">
+        <is>
+          <t>AJ Bell Great South Run</t>
+        </is>
+      </c>
+      <c r="B377" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C377" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D377" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E377" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="8" t="inlineStr">
+        <is>
+          <t>Army Ten Miler</t>
+        </is>
+      </c>
+      <c r="B378" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C378" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D378" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E378" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="4" t="inlineStr">
+        <is>
+          <t>Bay to Breakers</t>
+        </is>
+      </c>
+      <c r="B379" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C379" s="5" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D379" s="5" t="inlineStr">
+        <is>
+          <t>0:35:01</t>
+        </is>
+      </c>
+      <c r="E379" s="5" t="inlineStr">
+        <is>
+          <t>0:39:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="8" t="inlineStr">
+        <is>
+          <t>Bay to Breakers</t>
+        </is>
+      </c>
+      <c r="B380" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C380" s="9" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D380" s="9" t="inlineStr">
+        <is>
+          <t>0:36:10</t>
+        </is>
+      </c>
+      <c r="E380" s="9" t="inlineStr">
+        <is>
+          <t>0:42:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="4" t="inlineStr">
+        <is>
+          <t>Bay to Breakers</t>
+        </is>
+      </c>
+      <c r="B381" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C381" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D381" s="5" t="inlineStr">
+        <is>
+          <t>0:37:02</t>
+        </is>
+      </c>
+      <c r="E381" s="5" t="inlineStr">
+        <is>
+          <t>0:43:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="8" t="inlineStr">
+        <is>
+          <t>Boilermaker Road Race</t>
+        </is>
+      </c>
+      <c r="B382" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C382" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D382" s="9" t="inlineStr">
+        <is>
+          <t>0:42:44</t>
+        </is>
+      </c>
+      <c r="E382" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="4" t="inlineStr">
+        <is>
+          <t>Broad Street Run</t>
+        </is>
+      </c>
+      <c r="B383" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C383" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D383" s="5" t="inlineStr">
+        <is>
+          <t>0:46:13</t>
+        </is>
+      </c>
+      <c r="E383" s="5" t="inlineStr">
+        <is>
+          <t>0:54:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="8" t="inlineStr">
+        <is>
+          <t>City2Surf</t>
+        </is>
+      </c>
+      <c r="B384" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C384" s="9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D384" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E384" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="4" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B385" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C385" s="5" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D385" s="5" t="inlineStr">
+        <is>
+          <t>0:45:15</t>
+        </is>
+      </c>
+      <c r="E385" s="5" t="inlineStr">
+        <is>
+          <t>0:50:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="8" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B386" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C386" s="9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D386" s="9" t="inlineStr">
+        <is>
+          <t>0:44:51</t>
+        </is>
+      </c>
+      <c r="E386" s="9" t="inlineStr">
+        <is>
+          <t>0:51:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="4" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B387" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C387" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D387" s="5" t="inlineStr">
+        <is>
+          <t>0:46:07</t>
+        </is>
+      </c>
+      <c r="E387" s="5" t="inlineStr">
+        <is>
+          <t>0:50:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="8" t="inlineStr">
+        <is>
+          <t>Falmouth Road Race</t>
+        </is>
+      </c>
+      <c r="B388" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C388" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D388" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E388" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="4" t="inlineStr">
+        <is>
+          <t>Great Scottish Run</t>
+        </is>
+      </c>
+      <c r="B389" s="5" t="inlineStr">
+        <is>
+          <t>SEMI</t>
+        </is>
+      </c>
+      <c r="C389" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D389" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E389" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="8" t="inlineStr">
+        <is>
+          <t>Lilac Bloomsday Run</t>
+        </is>
+      </c>
+      <c r="B390" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C390" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D390" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E390" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="4" t="inlineStr">
+        <is>
+          <t>Manchester Road Race</t>
+        </is>
+      </c>
+      <c r="B391" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C391" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D391" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E391" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E366"/>
+  <autoFilter ref="A1:E391"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix wrong winner times for Great Manchester Run half marathon
The 21K entry for AJ Bell Great Manchester Run 2021 had 10-mile times
(0:52:12 / 0:57:46) instead of actual half marathon times.
Corrected to 1:10:25 (Luke Cotter) / 1:21:56 (Nicola Jackson).

This fixes the semi-marathon records display in Winners Times tab.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -16178,12 +16178,12 @@
       </c>
       <c r="D628" s="7" t="inlineStr">
         <is>
-          <t>0:52:12</t>
+          <t>1:10:25</t>
         </is>
       </c>
       <c r="E628" s="7" t="inlineStr">
         <is>
-          <t>0:57:46</t>
+          <t>1:21:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Marathon de Paris 2026: temps officiels API TimeTo + temps moyen
- Vainqueurs corrigés depuis API: H 2:05:18 (Crippa) / F 2:18:35 (Demise)
- Temps moyen général: 4:13:24 (57 396 finishers, 9.99 km/h)
- Ajout avg_times_sporthive.json + regeneration dashboard

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$908</definedName>
@@ -11228,12 +11228,12 @@
       </c>
       <c r="D430" s="3" t="inlineStr">
         <is>
-          <t>2:05:16</t>
+          <t>2:05:18</t>
         </is>
       </c>
       <c r="E430" s="3" t="inlineStr">
         <is>
-          <t>2:18:34</t>
+          <t>2:18:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto Update 4D 2026-05-12 — 1 update(s)
</commit_message>
<xml_diff>
--- a/Chronos_Vainqueurs.xlsx
+++ b/Chronos_Vainqueurs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Chronos Vainqueurs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$919</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chronos Vainqueurs'!$A$1:$E$937</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E919"/>
+  <dimension ref="A1:E937"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -19524,23 +19524,23 @@
         </is>
       </c>
       <c r="C762" s="7" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="D762" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:03:58</t>
         </is>
       </c>
       <c r="E762" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:12:54</t>
         </is>
       </c>
     </row>
     <row r="763">
       <c r="A763" s="4" t="inlineStr">
         <is>
-          <t>Nike Melbourne Marathon Festival</t>
+          <t>NYRR RBC Brooklyn Half</t>
         </is>
       </c>
       <c r="B763" s="5" t="inlineStr">
@@ -19549,23 +19549,23 @@
         </is>
       </c>
       <c r="C763" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D763" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:03:05</t>
         </is>
       </c>
       <c r="E763" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:11:38</t>
         </is>
       </c>
     </row>
     <row r="764">
       <c r="A764" s="6" t="inlineStr">
         <is>
-          <t>Riyadh Marathon (Half)</t>
+          <t>NYRR RBC Brooklyn Half</t>
         </is>
       </c>
       <c r="B764" s="7" t="inlineStr">
@@ -19574,23 +19574,23 @@
         </is>
       </c>
       <c r="C764" s="7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D764" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:08</t>
         </is>
       </c>
       <c r="E764" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:12:41</t>
         </is>
       </c>
     </row>
     <row r="765">
       <c r="A765" s="4" t="inlineStr">
         <is>
-          <t>Riyadh Marathon (Half)</t>
+          <t>NYRR RBC Brooklyn Half</t>
         </is>
       </c>
       <c r="B765" s="5" t="inlineStr">
@@ -19599,7 +19599,7 @@
         </is>
       </c>
       <c r="C765" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D765" s="5" t="inlineStr">
         <is>
@@ -19615,7 +19615,7 @@
     <row r="766">
       <c r="A766" s="6" t="inlineStr">
         <is>
-          <t>Riyadh Marathon (Half)</t>
+          <t>Nike Melbourne Marathon Festival</t>
         </is>
       </c>
       <c r="B766" s="7" t="inlineStr">
@@ -19649,7 +19649,7 @@
         </is>
       </c>
       <c r="C767" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D767" s="5" t="inlineStr">
         <is>
@@ -19665,7 +19665,7 @@
     <row r="768">
       <c r="A768" s="6" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Las Vegas</t>
+          <t>Riyadh Marathon (Half)</t>
         </is>
       </c>
       <c r="B768" s="7" t="inlineStr">
@@ -19674,7 +19674,7 @@
         </is>
       </c>
       <c r="C768" s="7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D768" s="7" t="inlineStr">
         <is>
@@ -19690,7 +19690,7 @@
     <row r="769">
       <c r="A769" s="4" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Las Vegas</t>
+          <t>Riyadh Marathon (Half)</t>
         </is>
       </c>
       <c r="B769" s="5" t="inlineStr">
@@ -19699,7 +19699,7 @@
         </is>
       </c>
       <c r="C769" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D769" s="5" t="inlineStr">
         <is>
@@ -19715,7 +19715,7 @@
     <row r="770">
       <c r="A770" s="6" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Las Vegas</t>
+          <t>Riyadh Marathon (Half)</t>
         </is>
       </c>
       <c r="B770" s="7" t="inlineStr">
@@ -19724,7 +19724,7 @@
         </is>
       </c>
       <c r="C770" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D770" s="7" t="inlineStr">
         <is>
@@ -19749,7 +19749,7 @@
         </is>
       </c>
       <c r="C771" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D771" s="5" t="inlineStr">
         <is>
@@ -19765,7 +19765,7 @@
     <row r="772">
       <c r="A772" s="6" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series Mexico City</t>
+          <t>Rock 'n' Roll Running Series Las Vegas</t>
         </is>
       </c>
       <c r="B772" s="7" t="inlineStr">
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="C772" s="7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D772" s="7" t="inlineStr">
         <is>
@@ -19790,7 +19790,7 @@
     <row r="773">
       <c r="A773" s="4" t="inlineStr">
         <is>
-          <t>Rock 'n' Roll Running Series San Diego</t>
+          <t>Rock 'n' Roll Running Series Las Vegas</t>
         </is>
       </c>
       <c r="B773" s="5" t="inlineStr">
@@ -19815,7 +19815,7 @@
     <row r="774">
       <c r="A774" s="6" t="inlineStr">
         <is>
-          <t>Royal Parks Half Marathon</t>
+          <t>Rock 'n' Roll Running Series Las Vegas</t>
         </is>
       </c>
       <c r="B774" s="7" t="inlineStr">
@@ -19824,7 +19824,7 @@
         </is>
       </c>
       <c r="C774" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D774" s="7" t="inlineStr">
         <is>
@@ -19840,7 +19840,7 @@
     <row r="775">
       <c r="A775" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (Semi)</t>
+          <t>Rock 'n' Roll Running Series Mexico City</t>
         </is>
       </c>
       <c r="B775" s="5" t="inlineStr">
@@ -19849,7 +19849,7 @@
         </is>
       </c>
       <c r="C775" s="5" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D775" s="5" t="inlineStr">
         <is>
@@ -19865,7 +19865,7 @@
     <row r="776">
       <c r="A776" s="6" t="inlineStr">
         <is>
-          <t>Run in Lyon (Semi)</t>
+          <t>Rock 'n' Roll Running Series San Diego</t>
         </is>
       </c>
       <c r="B776" s="7" t="inlineStr">
@@ -19874,23 +19874,23 @@
         </is>
       </c>
       <c r="C776" s="7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D776" s="7" t="inlineStr">
         <is>
-          <t>1:05:44</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E776" s="7" t="inlineStr">
         <is>
-          <t>1:18:34</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="777">
       <c r="A777" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (Semi)</t>
+          <t>Royal Parks Half Marathon</t>
         </is>
       </c>
       <c r="B777" s="5" t="inlineStr">
@@ -19915,7 +19915,7 @@
     <row r="778">
       <c r="A778" s="6" t="inlineStr">
         <is>
-          <t>Semi-Marathon de Boulogne-Billancourt</t>
+          <t>Run in Lyon (Semi)</t>
         </is>
       </c>
       <c r="B778" s="7" t="inlineStr">
@@ -19924,7 +19924,7 @@
         </is>
       </c>
       <c r="C778" s="7" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D778" s="7" t="inlineStr">
         <is>
@@ -19940,7 +19940,7 @@
     <row r="779">
       <c r="A779" s="4" t="inlineStr">
         <is>
-          <t>St. Jude Rock 'n' Roll Running Series Washington DC</t>
+          <t>Run in Lyon (Semi)</t>
         </is>
       </c>
       <c r="B779" s="5" t="inlineStr">
@@ -19949,23 +19949,23 @@
         </is>
       </c>
       <c r="C779" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D779" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:05:44</t>
         </is>
       </c>
       <c r="E779" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:18:34</t>
         </is>
       </c>
     </row>
     <row r="780">
       <c r="A780" s="6" t="inlineStr">
         <is>
-          <t>St. Jude Rock 'n' Roll Series Nashville</t>
+          <t>Run in Lyon (Semi)</t>
         </is>
       </c>
       <c r="B780" s="7" t="inlineStr">
@@ -19990,7 +19990,7 @@
     <row r="781">
       <c r="A781" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered Hong Kong Half Marathon</t>
+          <t>Semi-Marathon de Boulogne-Billancourt</t>
         </is>
       </c>
       <c r="B781" s="5" t="inlineStr">
@@ -19999,23 +19999,23 @@
         </is>
       </c>
       <c r="C781" s="5" t="n">
-        <v>2019</v>
+        <v>2025</v>
       </c>
       <c r="D781" s="5" t="inlineStr">
         <is>
-          <t>1:01:13</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E781" s="5" t="inlineStr">
         <is>
-          <t>1:09:28</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="782">
       <c r="A782" s="6" t="inlineStr">
         <is>
-          <t>Standard Chartered Hong Kong Half Marathon</t>
+          <t>St. Jude Rock 'n' Roll Running Series Washington DC</t>
         </is>
       </c>
       <c r="B782" s="7" t="inlineStr">
@@ -20040,7 +20040,7 @@
     <row r="783">
       <c r="A783" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered Hong Kong Half Marathon</t>
+          <t>St. Jude Rock 'n' Roll Series Nashville</t>
         </is>
       </c>
       <c r="B783" s="5" t="inlineStr">
@@ -20049,7 +20049,7 @@
         </is>
       </c>
       <c r="C783" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D783" s="5" t="inlineStr">
         <is>
@@ -20065,7 +20065,7 @@
     <row r="784">
       <c r="A784" s="6" t="inlineStr">
         <is>
-          <t>Standard Chartered KL Half Marathon</t>
+          <t>Standard Chartered Hong Kong Half Marathon</t>
         </is>
       </c>
       <c r="B784" s="7" t="inlineStr">
@@ -20074,23 +20074,23 @@
         </is>
       </c>
       <c r="C784" s="7" t="n">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="D784" s="7" t="inlineStr">
         <is>
-          <t>1:11:08</t>
+          <t>1:01:13</t>
         </is>
       </c>
       <c r="E784" s="7" t="inlineStr">
         <is>
-          <t>1:23:55</t>
+          <t>1:09:28</t>
         </is>
       </c>
     </row>
     <row r="785">
       <c r="A785" s="4" t="inlineStr">
         <is>
-          <t>Standard Chartered Singapore Half Marathon</t>
+          <t>Standard Chartered Hong Kong Half Marathon</t>
         </is>
       </c>
       <c r="B785" s="5" t="inlineStr">
@@ -20115,7 +20115,7 @@
     <row r="786">
       <c r="A786" s="6" t="inlineStr">
         <is>
-          <t>TCS Mizuno Half Marathon</t>
+          <t>Standard Chartered Hong Kong Half Marathon</t>
         </is>
       </c>
       <c r="B786" s="7" t="inlineStr">
@@ -20124,23 +20124,23 @@
         </is>
       </c>
       <c r="C786" s="7" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D786" s="7" t="inlineStr">
         <is>
-          <t>1:05:23</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E786" s="7" t="inlineStr">
         <is>
-          <t>1:13:59</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="787">
       <c r="A787" s="4" t="inlineStr">
         <is>
-          <t>TCS Mizuno Half Marathon</t>
+          <t>Standard Chartered KL Half Marathon</t>
         </is>
       </c>
       <c r="B787" s="5" t="inlineStr">
@@ -20149,23 +20149,23 @@
         </is>
       </c>
       <c r="C787" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D787" s="5" t="inlineStr">
         <is>
-          <t>1:06:28</t>
+          <t>1:11:08</t>
         </is>
       </c>
       <c r="E787" s="5" t="inlineStr">
         <is>
-          <t>1:17:54</t>
+          <t>1:23:55</t>
         </is>
       </c>
     </row>
     <row r="788">
       <c r="A788" s="6" t="inlineStr">
         <is>
-          <t>TCS Mizuno Half Marathon</t>
+          <t>Standard Chartered Singapore Half Marathon</t>
         </is>
       </c>
       <c r="B788" s="7" t="inlineStr">
@@ -20199,23 +20199,23 @@
         </is>
       </c>
       <c r="C789" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D789" s="5" t="inlineStr">
         <is>
-          <t>1:04:21</t>
+          <t>1:05:23</t>
         </is>
       </c>
       <c r="E789" s="5" t="inlineStr">
         <is>
-          <t>1:10:02</t>
+          <t>1:13:59</t>
         </is>
       </c>
     </row>
     <row r="790">
       <c r="A790" s="6" t="inlineStr">
         <is>
-          <t>TCS Toronto Waterfront Marathon (Half)</t>
+          <t>TCS Mizuno Half Marathon</t>
         </is>
       </c>
       <c r="B790" s="7" t="inlineStr">
@@ -20224,23 +20224,23 @@
         </is>
       </c>
       <c r="C790" s="7" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D790" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:28</t>
         </is>
       </c>
       <c r="E790" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:17:54</t>
         </is>
       </c>
     </row>
     <row r="791">
       <c r="A791" s="4" t="inlineStr">
         <is>
-          <t>TCS Toronto Waterfront Marathon (Half)</t>
+          <t>TCS Mizuno Half Marathon</t>
         </is>
       </c>
       <c r="B791" s="5" t="inlineStr">
@@ -20249,7 +20249,7 @@
         </is>
       </c>
       <c r="C791" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D791" s="5" t="inlineStr">
         <is>
@@ -20265,7 +20265,7 @@
     <row r="792">
       <c r="A792" s="6" t="inlineStr">
         <is>
-          <t>TCS Toronto Waterfront Marathon (Half)</t>
+          <t>TCS Mizuno Half Marathon</t>
         </is>
       </c>
       <c r="B792" s="7" t="inlineStr">
@@ -20278,19 +20278,19 @@
       </c>
       <c r="D792" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:04:21</t>
         </is>
       </c>
       <c r="E792" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:10:02</t>
         </is>
       </c>
     </row>
     <row r="793">
       <c r="A793" s="4" t="inlineStr">
         <is>
-          <t>Taipei Half Marathon</t>
+          <t>TCS Toronto Waterfront Marathon (Half)</t>
         </is>
       </c>
       <c r="B793" s="5" t="inlineStr">
@@ -20315,7 +20315,7 @@
     <row r="794">
       <c r="A794" s="6" t="inlineStr">
         <is>
-          <t>Taipei Half Marathon</t>
+          <t>TCS Toronto Waterfront Marathon (Half)</t>
         </is>
       </c>
       <c r="B794" s="7" t="inlineStr">
@@ -20340,7 +20340,7 @@
     <row r="795">
       <c r="A795" s="4" t="inlineStr">
         <is>
-          <t>Taipei Half Marathon</t>
+          <t>TCS Toronto Waterfront Marathon (Half)</t>
         </is>
       </c>
       <c r="B795" s="5" t="inlineStr">
@@ -20365,7 +20365,7 @@
     <row r="796">
       <c r="A796" s="6" t="inlineStr">
         <is>
-          <t>Tata Mumbai Marathon (Half)</t>
+          <t>Taipei Half Marathon</t>
         </is>
       </c>
       <c r="B796" s="7" t="inlineStr">
@@ -20374,7 +20374,7 @@
         </is>
       </c>
       <c r="C796" s="7" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D796" s="7" t="inlineStr">
         <is>
@@ -20390,7 +20390,7 @@
     <row r="797">
       <c r="A797" s="4" t="inlineStr">
         <is>
-          <t>Tata Mumbai Marathon (Half)</t>
+          <t>Taipei Half Marathon</t>
         </is>
       </c>
       <c r="B797" s="5" t="inlineStr">
@@ -20399,7 +20399,7 @@
         </is>
       </c>
       <c r="C797" s="5" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D797" s="5" t="inlineStr">
         <is>
@@ -20415,7 +20415,7 @@
     <row r="798">
       <c r="A798" s="6" t="inlineStr">
         <is>
-          <t>The Big Half</t>
+          <t>Taipei Half Marathon</t>
         </is>
       </c>
       <c r="B798" s="7" t="inlineStr">
@@ -20440,7 +20440,7 @@
     <row r="799">
       <c r="A799" s="4" t="inlineStr">
         <is>
-          <t>Tokyo Legacy Half Marathon</t>
+          <t>Tata Mumbai Marathon (Half)</t>
         </is>
       </c>
       <c r="B799" s="5" t="inlineStr">
@@ -20465,7 +20465,7 @@
     <row r="800">
       <c r="A800" s="6" t="inlineStr">
         <is>
-          <t>United Airlines NYC Half</t>
+          <t>Tata Mumbai Marathon (Half)</t>
         </is>
       </c>
       <c r="B800" s="7" t="inlineStr">
@@ -20474,23 +20474,23 @@
         </is>
       </c>
       <c r="C800" s="7" t="n">
-        <v>2006</v>
+        <v>2026</v>
       </c>
       <c r="D800" s="7" t="inlineStr">
         <is>
-          <t>1:01:22</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E800" s="7" t="inlineStr">
         <is>
-          <t>1:09:43</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="801">
       <c r="A801" s="4" t="inlineStr">
         <is>
-          <t>United Airlines NYC Half</t>
+          <t>The Big Half</t>
         </is>
       </c>
       <c r="B801" s="5" t="inlineStr">
@@ -20499,23 +20499,23 @@
         </is>
       </c>
       <c r="C801" s="5" t="n">
-        <v>2007</v>
+        <v>2025</v>
       </c>
       <c r="D801" s="5" t="inlineStr">
         <is>
-          <t>0:59:24</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E801" s="5" t="inlineStr">
         <is>
-          <t>1:10:32</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="802">
       <c r="A802" s="6" t="inlineStr">
         <is>
-          <t>United Airlines NYC Half</t>
+          <t>Tokyo Legacy Half Marathon</t>
         </is>
       </c>
       <c r="B802" s="7" t="inlineStr">
@@ -20524,16 +20524,16 @@
         </is>
       </c>
       <c r="C802" s="7" t="n">
-        <v>2008</v>
+        <v>2025</v>
       </c>
       <c r="D802" s="7" t="inlineStr">
         <is>
-          <t>1:00:58</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E802" s="7" t="inlineStr">
         <is>
-          <t>1:10:19</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -20549,16 +20549,16 @@
         </is>
       </c>
       <c r="C803" s="5" t="n">
-        <v>2009</v>
+        <v>2006</v>
       </c>
       <c r="D803" s="5" t="inlineStr">
         <is>
-          <t>1:01:06</t>
+          <t>1:01:22</t>
         </is>
       </c>
       <c r="E803" s="5" t="inlineStr">
         <is>
-          <t>1:09:32</t>
+          <t>1:09:43</t>
         </is>
       </c>
     </row>
@@ -20574,16 +20574,16 @@
         </is>
       </c>
       <c r="C804" s="7" t="n">
-        <v>2010</v>
+        <v>2007</v>
       </c>
       <c r="D804" s="7" t="inlineStr">
         <is>
-          <t>0:59:52</t>
+          <t>0:59:24</t>
         </is>
       </c>
       <c r="E804" s="7" t="inlineStr">
         <is>
-          <t>1:09:25</t>
+          <t>1:10:32</t>
         </is>
       </c>
     </row>
@@ -20599,16 +20599,16 @@
         </is>
       </c>
       <c r="C805" s="5" t="n">
-        <v>2011</v>
+        <v>2008</v>
       </c>
       <c r="D805" s="5" t="inlineStr">
         <is>
-          <t>1:00:23</t>
+          <t>1:00:58</t>
         </is>
       </c>
       <c r="E805" s="5" t="inlineStr">
         <is>
-          <t>1:08:52</t>
+          <t>1:10:19</t>
         </is>
       </c>
     </row>
@@ -20624,16 +20624,16 @@
         </is>
       </c>
       <c r="C806" s="7" t="n">
-        <v>2012</v>
+        <v>2009</v>
       </c>
       <c r="D806" s="7" t="inlineStr">
         <is>
-          <t>0:59:39</t>
+          <t>1:01:06</t>
         </is>
       </c>
       <c r="E806" s="7" t="inlineStr">
         <is>
-          <t>1:08:35</t>
+          <t>1:09:32</t>
         </is>
       </c>
     </row>
@@ -20649,16 +20649,16 @@
         </is>
       </c>
       <c r="C807" s="5" t="n">
-        <v>2013</v>
+        <v>2010</v>
       </c>
       <c r="D807" s="5" t="inlineStr">
         <is>
-          <t>1:01:02</t>
+          <t>0:59:52</t>
         </is>
       </c>
       <c r="E807" s="5" t="inlineStr">
         <is>
-          <t>1:09:09</t>
+          <t>1:09:25</t>
         </is>
       </c>
     </row>
@@ -20674,16 +20674,16 @@
         </is>
       </c>
       <c r="C808" s="7" t="n">
-        <v>2014</v>
+        <v>2011</v>
       </c>
       <c r="D808" s="7" t="inlineStr">
         <is>
-          <t>1:00:50</t>
+          <t>1:00:23</t>
         </is>
       </c>
       <c r="E808" s="7" t="inlineStr">
         <is>
-          <t>1:08:31</t>
+          <t>1:08:52</t>
         </is>
       </c>
     </row>
@@ -20699,16 +20699,16 @@
         </is>
       </c>
       <c r="C809" s="5" t="n">
-        <v>2025</v>
+        <v>2012</v>
       </c>
       <c r="D809" s="5" t="inlineStr">
         <is>
-          <t>1:01:31</t>
+          <t>0:59:39</t>
         </is>
       </c>
       <c r="E809" s="5" t="inlineStr">
         <is>
-          <t>1:07:04</t>
+          <t>1:08:35</t>
         </is>
       </c>
     </row>
@@ -20724,23 +20724,23 @@
         </is>
       </c>
       <c r="C810" s="7" t="n">
-        <v>2026</v>
+        <v>2013</v>
       </c>
       <c r="D810" s="7" t="inlineStr">
         <is>
-          <t>0:59:30</t>
+          <t>1:01:02</t>
         </is>
       </c>
       <c r="E810" s="7" t="inlineStr">
         <is>
-          <t>1:06:33</t>
+          <t>1:09:09</t>
         </is>
       </c>
     </row>
     <row r="811">
       <c r="A811" s="4" t="inlineStr">
         <is>
-          <t>Valencia Half Marathon Trinidad Alfonso Zurich</t>
+          <t>United Airlines NYC Half</t>
         </is>
       </c>
       <c r="B811" s="5" t="inlineStr">
@@ -20749,23 +20749,23 @@
         </is>
       </c>
       <c r="C811" s="5" t="n">
-        <v>2025</v>
+        <v>2014</v>
       </c>
       <c r="D811" s="5" t="inlineStr">
         <is>
-          <t>0:58:02</t>
+          <t>1:00:50</t>
         </is>
       </c>
       <c r="E811" s="5" t="inlineStr">
         <is>
-          <t>1:03:08</t>
+          <t>1:08:31</t>
         </is>
       </c>
     </row>
     <row r="812">
       <c r="A812" s="6" t="inlineStr">
         <is>
-          <t>Vedanta Delhi Half Marathon</t>
+          <t>United Airlines NYC Half</t>
         </is>
       </c>
       <c r="B812" s="7" t="inlineStr">
@@ -20778,19 +20778,19 @@
       </c>
       <c r="D812" s="7" t="inlineStr">
         <is>
-          <t>0:59:50</t>
+          <t>1:01:31</t>
         </is>
       </c>
       <c r="E812" s="7" t="inlineStr">
         <is>
-          <t>1:07:20</t>
+          <t>1:07:04</t>
         </is>
       </c>
     </row>
     <row r="813">
       <c r="A813" s="4" t="inlineStr">
         <is>
-          <t>Vienna City Half Marathon</t>
+          <t>United Airlines NYC Half</t>
         </is>
       </c>
       <c r="B813" s="5" t="inlineStr">
@@ -20799,23 +20799,23 @@
         </is>
       </c>
       <c r="C813" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D813" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:30</t>
         </is>
       </c>
       <c r="E813" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:06:33</t>
         </is>
       </c>
     </row>
     <row r="814">
       <c r="A814" s="6" t="inlineStr">
         <is>
-          <t>Walt Disney World Marathon Weekend</t>
+          <t>Valencia Half Marathon Trinidad Alfonso Zurich</t>
         </is>
       </c>
       <c r="B814" s="7" t="inlineStr">
@@ -20828,19 +20828,19 @@
       </c>
       <c r="D814" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:58:02</t>
         </is>
       </c>
       <c r="E814" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:03:08</t>
         </is>
       </c>
     </row>
     <row r="815">
       <c r="A815" s="4" t="inlineStr">
         <is>
-          <t>Walt Disney World Marathon Weekend</t>
+          <t>Vedanta Delhi Half Marathon</t>
         </is>
       </c>
       <c r="B815" s="5" t="inlineStr">
@@ -20849,23 +20849,23 @@
         </is>
       </c>
       <c r="C815" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D815" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:50</t>
         </is>
       </c>
       <c r="E815" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:07:20</t>
         </is>
       </c>
     </row>
     <row r="816">
       <c r="A816" s="6" t="inlineStr">
         <is>
-          <t>Warsaw Half Marathon</t>
+          <t>Vienna City Half Marathon</t>
         </is>
       </c>
       <c r="B816" s="7" t="inlineStr">
@@ -20874,7 +20874,7 @@
         </is>
       </c>
       <c r="C816" s="7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D816" s="7" t="inlineStr">
         <is>
@@ -20890,7 +20890,7 @@
     <row r="817">
       <c r="A817" s="4" t="inlineStr">
         <is>
-          <t>Warsaw Half Marathon</t>
+          <t>Walt Disney World Marathon Weekend</t>
         </is>
       </c>
       <c r="B817" s="5" t="inlineStr">
@@ -20915,7 +20915,7 @@
     <row r="818">
       <c r="A818" s="6" t="inlineStr">
         <is>
-          <t>Wizz Air Rome Half Marathon by Brooks</t>
+          <t>Walt Disney World Marathon Weekend</t>
         </is>
       </c>
       <c r="B818" s="7" t="inlineStr">
@@ -20924,7 +20924,7 @@
         </is>
       </c>
       <c r="C818" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D818" s="7" t="inlineStr">
         <is>
@@ -20940,7 +20940,7 @@
     <row r="819">
       <c r="A819" s="4" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+          <t>Warsaw Half Marathon</t>
         </is>
       </c>
       <c r="B819" s="5" t="inlineStr">
@@ -20949,7 +20949,7 @@
         </is>
       </c>
       <c r="C819" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D819" s="5" t="inlineStr">
         <is>
@@ -20965,7 +20965,7 @@
     <row r="820">
       <c r="A820" s="6" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+          <t>Warsaw Half Marathon</t>
         </is>
       </c>
       <c r="B820" s="7" t="inlineStr">
@@ -20974,7 +20974,7 @@
         </is>
       </c>
       <c r="C820" s="7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D820" s="7" t="inlineStr">
         <is>
@@ -20990,7 +20990,7 @@
     <row r="821">
       <c r="A821" s="4" t="inlineStr">
         <is>
-          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+          <t>Wizz Air Rome Half Marathon by Brooks</t>
         </is>
       </c>
       <c r="B821" s="5" t="inlineStr">
@@ -21013,43 +21013,43 @@
       </c>
     </row>
     <row r="822">
-      <c r="A822" s="8" t="inlineStr">
-        <is>
-          <t>10K Montmartre</t>
-        </is>
-      </c>
-      <c r="B822" s="9" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
-      <c r="C822" s="9" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D822" s="9" t="inlineStr">
-        <is>
-          <t>0:31:14</t>
-        </is>
-      </c>
-      <c r="E822" s="9" t="inlineStr">
-        <is>
-          <t>0:35:46</t>
+      <c r="A822" s="6" t="inlineStr">
+        <is>
+          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+        </is>
+      </c>
+      <c r="B822" s="7" t="inlineStr">
+        <is>
+          <t>21K</t>
+        </is>
+      </c>
+      <c r="C822" s="7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D822" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E822" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="823">
       <c r="A823" s="4" t="inlineStr">
         <is>
-          <t>10K Montmartre</t>
+          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
         </is>
       </c>
       <c r="B823" s="5" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>21K</t>
         </is>
       </c>
       <c r="C823" s="5" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D823" s="5" t="inlineStr">
         <is>
@@ -21063,34 +21063,34 @@
       </c>
     </row>
     <row r="824">
-      <c r="A824" s="8" t="inlineStr">
-        <is>
-          <t>10K Valencia Ibercaja by Kiprun</t>
-        </is>
-      </c>
-      <c r="B824" s="9" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
-      <c r="C824" s="9" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D824" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E824" s="9" t="inlineStr">
-        <is>
-          <t>0:29:19</t>
+      <c r="A824" s="6" t="inlineStr">
+        <is>
+          <t>Zurich Rock 'n' Roll Running Series Madrid (Half)</t>
+        </is>
+      </c>
+      <c r="B824" s="7" t="inlineStr">
+        <is>
+          <t>21K</t>
+        </is>
+      </c>
+      <c r="C824" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D824" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E824" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="825">
       <c r="A825" s="4" t="inlineStr">
         <is>
-          <t>10K Valencia Ibercaja by Kiprun</t>
+          <t>10K Montmartre</t>
         </is>
       </c>
       <c r="B825" s="5" t="inlineStr">
@@ -21099,23 +21099,23 @@
         </is>
       </c>
       <c r="C825" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D825" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:14</t>
         </is>
       </c>
       <c r="E825" s="5" t="inlineStr">
         <is>
-          <t>0:28:45</t>
+          <t>0:35:46</t>
         </is>
       </c>
     </row>
     <row r="826">
       <c r="A826" s="8" t="inlineStr">
         <is>
-          <t>10K Valencia Ibercaja by Kiprun</t>
+          <t>10K Montmartre</t>
         </is>
       </c>
       <c r="B826" s="9" t="inlineStr">
@@ -21124,7 +21124,7 @@
         </is>
       </c>
       <c r="C826" s="9" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D826" s="9" t="inlineStr">
         <is>
@@ -21149,23 +21149,23 @@
         </is>
       </c>
       <c r="C827" s="5" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D827" s="5" t="inlineStr">
         <is>
-          <t>0:26:45</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E827" s="5" t="inlineStr">
         <is>
-          <t>0:29:25</t>
+          <t>0:29:19</t>
         </is>
       </c>
     </row>
     <row r="828">
       <c r="A828" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Birmingham Run 10K</t>
+          <t>10K Valencia Ibercaja by Kiprun</t>
         </is>
       </c>
       <c r="B828" s="9" t="inlineStr">
@@ -21174,7 +21174,7 @@
         </is>
       </c>
       <c r="C828" s="9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D828" s="9" t="inlineStr">
         <is>
@@ -21183,14 +21183,14 @@
       </c>
       <c r="E828" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:45</t>
         </is>
       </c>
     </row>
     <row r="829">
       <c r="A829" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great Bristol Run 10K</t>
+          <t>10K Valencia Ibercaja by Kiprun</t>
         </is>
       </c>
       <c r="B829" s="5" t="inlineStr">
@@ -21215,7 +21215,7 @@
     <row r="830">
       <c r="A830" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run</t>
+          <t>10K Valencia Ibercaja by Kiprun</t>
         </is>
       </c>
       <c r="B830" s="9" t="inlineStr">
@@ -21224,23 +21224,23 @@
         </is>
       </c>
       <c r="C830" s="9" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="D830" s="9" t="inlineStr">
         <is>
-          <t>0:28:03</t>
+          <t>0:26:45</t>
         </is>
       </c>
       <c r="E830" s="9" t="inlineStr">
         <is>
-          <t>0:30:51</t>
+          <t>0:29:25</t>
         </is>
       </c>
     </row>
     <row r="831">
       <c r="A831" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run</t>
+          <t>AJ Bell Great Birmingham Run 10K</t>
         </is>
       </c>
       <c r="B831" s="5" t="inlineStr">
@@ -21265,7 +21265,7 @@
     <row r="832">
       <c r="A832" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run (10K)</t>
+          <t>AJ Bell Great Bristol Run 10K</t>
         </is>
       </c>
       <c r="B832" s="9" t="inlineStr">
@@ -21274,7 +21274,7 @@
         </is>
       </c>
       <c r="C832" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D832" s="9" t="inlineStr">
         <is>
@@ -21290,7 +21290,7 @@
     <row r="833">
       <c r="A833" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great Manchester Run (10K)</t>
+          <t>AJ Bell Great Manchester Run</t>
         </is>
       </c>
       <c r="B833" s="5" t="inlineStr">
@@ -21299,23 +21299,23 @@
         </is>
       </c>
       <c r="C833" s="5" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="D833" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:03</t>
         </is>
       </c>
       <c r="E833" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:30:51</t>
         </is>
       </c>
     </row>
     <row r="834">
       <c r="A834" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great North 10K</t>
+          <t>AJ Bell Great Manchester Run</t>
         </is>
       </c>
       <c r="B834" s="9" t="inlineStr">
@@ -21340,7 +21340,7 @@
     <row r="835">
       <c r="A835" s="4" t="inlineStr">
         <is>
-          <t>ASICS LDNX</t>
+          <t>AJ Bell Great Manchester Run (10K)</t>
         </is>
       </c>
       <c r="B835" s="5" t="inlineStr">
@@ -21349,7 +21349,7 @@
         </is>
       </c>
       <c r="C835" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D835" s="5" t="inlineStr">
         <is>
@@ -21365,7 +21365,7 @@
     <row r="836">
       <c r="A836" s="8" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>AJ Bell Great Manchester Run (10K)</t>
         </is>
       </c>
       <c r="B836" s="9" t="inlineStr">
@@ -21374,7 +21374,7 @@
         </is>
       </c>
       <c r="C836" s="9" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="D836" s="9" t="inlineStr">
         <is>
@@ -21390,7 +21390,7 @@
     <row r="837">
       <c r="A837" s="4" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>AJ Bell Great North 10K</t>
         </is>
       </c>
       <c r="B837" s="5" t="inlineStr">
@@ -21399,23 +21399,23 @@
         </is>
       </c>
       <c r="C837" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D837" s="5" t="inlineStr">
         <is>
-          <t>0:29:37</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E837" s="5" t="inlineStr">
         <is>
-          <t>0:32:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="838">
       <c r="A838" s="8" t="inlineStr">
         <is>
-          <t>Adidas 10K Paris</t>
+          <t>ASICS LDNX</t>
         </is>
       </c>
       <c r="B838" s="9" t="inlineStr">
@@ -21440,7 +21440,7 @@
     <row r="839">
       <c r="A839" s="4" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B839" s="5" t="inlineStr">
@@ -21453,19 +21453,19 @@
       </c>
       <c r="D839" s="5" t="inlineStr">
         <is>
-          <t>0:27:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E839" s="5" t="inlineStr">
         <is>
-          <t>0:30:43</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="840">
       <c r="A840" s="8" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B840" s="9" t="inlineStr">
@@ -21478,19 +21478,19 @@
       </c>
       <c r="D840" s="9" t="inlineStr">
         <is>
-          <t>0:28:03</t>
+          <t>0:29:37</t>
         </is>
       </c>
       <c r="E840" s="9" t="inlineStr">
         <is>
-          <t>0:31:12</t>
+          <t>0:32:18</t>
         </is>
       </c>
     </row>
     <row r="841">
       <c r="A841" s="4" t="inlineStr">
         <is>
-          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
+          <t>Adidas 10K Paris</t>
         </is>
       </c>
       <c r="B841" s="5" t="inlineStr">
@@ -21508,14 +21508,14 @@
       </c>
       <c r="E841" s="5" t="inlineStr">
         <is>
-          <t>0:31:29</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="842">
       <c r="A842" s="8" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B842" s="9" t="inlineStr">
@@ -21528,19 +21528,19 @@
       </c>
       <c r="D842" s="9" t="inlineStr">
         <is>
-          <t>0:29:08</t>
+          <t>0:27:41</t>
         </is>
       </c>
       <c r="E842" s="9" t="inlineStr">
         <is>
-          <t>0:33:25</t>
+          <t>0:30:43</t>
         </is>
       </c>
     </row>
     <row r="843">
       <c r="A843" s="4" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B843" s="5" t="inlineStr">
@@ -21553,19 +21553,19 @@
       </c>
       <c r="D843" s="5" t="inlineStr">
         <is>
-          <t>0:29:13</t>
+          <t>0:28:03</t>
         </is>
       </c>
       <c r="E843" s="5" t="inlineStr">
         <is>
-          <t>0:32:45</t>
+          <t>0:31:12</t>
         </is>
       </c>
     </row>
     <row r="844">
       <c r="A844" s="8" t="inlineStr">
         <is>
-          <t>BOLDERBoulder 10K</t>
+          <t>Atlanta Journal-Constitution Peachtree Road Race</t>
         </is>
       </c>
       <c r="B844" s="9" t="inlineStr">
@@ -21583,7 +21583,7 @@
       </c>
       <c r="E844" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:29</t>
         </is>
       </c>
     </row>
@@ -21599,23 +21599,23 @@
         </is>
       </c>
       <c r="C845" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D845" s="5" t="inlineStr">
         <is>
-          <t>0:28:36</t>
+          <t>0:29:08</t>
         </is>
       </c>
       <c r="E845" s="5" t="inlineStr">
         <is>
-          <t>0:31:51</t>
+          <t>0:33:25</t>
         </is>
       </c>
     </row>
     <row r="846">
       <c r="A846" s="8" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B846" s="9" t="inlineStr">
@@ -21624,23 +21624,23 @@
         </is>
       </c>
       <c r="C846" s="9" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D846" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:13</t>
         </is>
       </c>
       <c r="E846" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:45</t>
         </is>
       </c>
     </row>
     <row r="847">
       <c r="A847" s="4" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B847" s="5" t="inlineStr">
@@ -21649,7 +21649,7 @@
         </is>
       </c>
       <c r="C847" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D847" s="5" t="inlineStr">
         <is>
@@ -21665,7 +21665,7 @@
     <row r="848">
       <c r="A848" s="8" t="inlineStr">
         <is>
-          <t>Bangsaen10</t>
+          <t>BOLDERBoulder 10K</t>
         </is>
       </c>
       <c r="B848" s="9" t="inlineStr">
@@ -21678,19 +21678,19 @@
       </c>
       <c r="D848" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:36</t>
         </is>
       </c>
       <c r="E848" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:51</t>
         </is>
       </c>
     </row>
     <row r="849">
       <c r="A849" s="4" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B849" s="5" t="inlineStr">
@@ -21703,19 +21703,19 @@
       </c>
       <c r="D849" s="5" t="inlineStr">
         <is>
-          <t>0:28:52</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E849" s="5" t="inlineStr">
         <is>
-          <t>0:31:59</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="850">
       <c r="A850" s="8" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B850" s="9" t="inlineStr">
@@ -21728,19 +21728,19 @@
       </c>
       <c r="D850" s="9" t="inlineStr">
         <is>
-          <t>0:28:46</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E850" s="9" t="inlineStr">
         <is>
-          <t>0:32:33</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="851">
       <c r="A851" s="4" t="inlineStr">
         <is>
-          <t>Cancer Research UK London Winter Run</t>
+          <t>Bangsaen10</t>
         </is>
       </c>
       <c r="B851" s="5" t="inlineStr">
@@ -21753,12 +21753,12 @@
       </c>
       <c r="D851" s="5" t="inlineStr">
         <is>
-          <t>0:29:22</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E851" s="5" t="inlineStr">
         <is>
-          <t>0:34:32</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -21774,23 +21774,23 @@
         </is>
       </c>
       <c r="C852" s="9" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D852" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:52</t>
         </is>
       </c>
       <c r="E852" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:59</t>
         </is>
       </c>
     </row>
     <row r="853">
       <c r="A853" s="4" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B853" s="5" t="inlineStr">
@@ -21799,23 +21799,23 @@
         </is>
       </c>
       <c r="C853" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D853" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:46</t>
         </is>
       </c>
       <c r="E853" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:33</t>
         </is>
       </c>
     </row>
     <row r="854">
       <c r="A854" s="8" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B854" s="9" t="inlineStr">
@@ -21824,23 +21824,23 @@
         </is>
       </c>
       <c r="C854" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D854" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:22</t>
         </is>
       </c>
       <c r="E854" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:34:32</t>
         </is>
       </c>
     </row>
     <row r="855">
       <c r="A855" s="4" t="inlineStr">
         <is>
-          <t>Cooper River Bridge Run</t>
+          <t>Cancer Research UK London Winter Run</t>
         </is>
       </c>
       <c r="B855" s="5" t="inlineStr">
@@ -21849,16 +21849,16 @@
         </is>
       </c>
       <c r="C855" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D855" s="5" t="inlineStr">
         <is>
-          <t>0:28:27</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E855" s="5" t="inlineStr">
         <is>
-          <t>0:31:49</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -21874,7 +21874,7 @@
         </is>
       </c>
       <c r="C856" s="9" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D856" s="9" t="inlineStr">
         <is>
@@ -21890,7 +21890,7 @@
     <row r="857">
       <c r="A857" s="4" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B857" s="5" t="inlineStr">
@@ -21899,7 +21899,7 @@
         </is>
       </c>
       <c r="C857" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D857" s="5" t="inlineStr">
         <is>
@@ -21915,7 +21915,7 @@
     <row r="858">
       <c r="A858" s="8" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B858" s="9" t="inlineStr">
@@ -21924,23 +21924,23 @@
         </is>
       </c>
       <c r="C858" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D858" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:27</t>
         </is>
       </c>
       <c r="E858" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:49</t>
         </is>
       </c>
     </row>
     <row r="859">
       <c r="A859" s="4" t="inlineStr">
         <is>
-          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
+          <t>Cooper River Bridge Run</t>
         </is>
       </c>
       <c r="B859" s="5" t="inlineStr">
@@ -21974,7 +21974,7 @@
         </is>
       </c>
       <c r="C860" s="9" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="D860" s="9" t="inlineStr">
         <is>
@@ -21990,7 +21990,7 @@
     <row r="861">
       <c r="A861" s="4" t="inlineStr">
         <is>
-          <t>Great Scottish Run 10K</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B861" s="5" t="inlineStr">
@@ -21999,7 +21999,7 @@
         </is>
       </c>
       <c r="C861" s="5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D861" s="5" t="inlineStr">
         <is>
@@ -22015,7 +22015,7 @@
     <row r="862">
       <c r="A862" s="8" t="inlineStr">
         <is>
-          <t>NN CPC Loop Den Haag - 10 KM Loop</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B862" s="9" t="inlineStr">
@@ -22024,7 +22024,7 @@
         </is>
       </c>
       <c r="C862" s="9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D862" s="9" t="inlineStr">
         <is>
@@ -22040,7 +22040,7 @@
     <row r="863">
       <c r="A863" s="4" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>EDP Meia Maratona de Lisboa - Vodafone 10K</t>
         </is>
       </c>
       <c r="B863" s="5" t="inlineStr">
@@ -22049,7 +22049,7 @@
         </is>
       </c>
       <c r="C863" s="5" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D863" s="5" t="inlineStr">
         <is>
@@ -22065,7 +22065,7 @@
     <row r="864">
       <c r="A864" s="8" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>Great Scottish Run 10K</t>
         </is>
       </c>
       <c r="B864" s="9" t="inlineStr">
@@ -22074,7 +22074,7 @@
         </is>
       </c>
       <c r="C864" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D864" s="9" t="inlineStr">
         <is>
@@ -22083,14 +22083,14 @@
       </c>
       <c r="E864" s="9" t="inlineStr">
         <is>
-          <t>0:31:18</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="865">
       <c r="A865" s="4" t="inlineStr">
         <is>
-          <t>NN San Silvestre Vallecana</t>
+          <t>NN CPC Loop Den Haag - 10 KM Loop</t>
         </is>
       </c>
       <c r="B865" s="5" t="inlineStr">
@@ -22099,23 +22099,23 @@
         </is>
       </c>
       <c r="C865" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D865" s="5" t="inlineStr">
         <is>
-          <t>0:27:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E865" s="5" t="inlineStr">
         <is>
-          <t>0:31:11</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="866">
       <c r="A866" s="8" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B866" s="9" t="inlineStr">
@@ -22140,7 +22140,7 @@
     <row r="867">
       <c r="A867" s="4" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B867" s="5" t="inlineStr">
@@ -22158,14 +22158,14 @@
       </c>
       <c r="E867" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:18</t>
         </is>
       </c>
     </row>
     <row r="868">
       <c r="A868" s="8" t="inlineStr">
         <is>
-          <t>Royal Run</t>
+          <t>NN San Silvestre Vallecana</t>
         </is>
       </c>
       <c r="B868" s="9" t="inlineStr">
@@ -22178,19 +22178,19 @@
       </c>
       <c r="D868" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:27:41</t>
         </is>
       </c>
       <c r="E868" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:31:11</t>
         </is>
       </c>
     </row>
     <row r="869">
       <c r="A869" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B869" s="5" t="inlineStr">
@@ -22199,7 +22199,7 @@
         </is>
       </c>
       <c r="C869" s="5" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D869" s="5" t="inlineStr">
         <is>
@@ -22215,7 +22215,7 @@
     <row r="870">
       <c r="A870" s="8" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B870" s="9" t="inlineStr">
@@ -22224,7 +22224,7 @@
         </is>
       </c>
       <c r="C870" s="9" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D870" s="9" t="inlineStr">
         <is>
@@ -22240,7 +22240,7 @@
     <row r="871">
       <c r="A871" s="4" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>Royal Run</t>
         </is>
       </c>
       <c r="B871" s="5" t="inlineStr">
@@ -22249,7 +22249,7 @@
         </is>
       </c>
       <c r="C871" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D871" s="5" t="inlineStr">
         <is>
@@ -22265,7 +22265,7 @@
     <row r="872">
       <c r="A872" s="8" t="inlineStr">
         <is>
-          <t>Run in Lyon (10K)</t>
+          <t>Run in Lyon</t>
         </is>
       </c>
       <c r="B872" s="9" t="inlineStr">
@@ -22290,7 +22290,7 @@
     <row r="873">
       <c r="A873" s="4" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B873" s="5" t="inlineStr">
@@ -22315,7 +22315,7 @@
     <row r="874">
       <c r="A874" s="8" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B874" s="9" t="inlineStr">
@@ -22328,19 +22328,19 @@
       </c>
       <c r="D874" s="9" t="inlineStr">
         <is>
-          <t>0:29:41</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E874" s="9" t="inlineStr">
         <is>
-          <t>0:32:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="875">
       <c r="A875" s="4" t="inlineStr">
         <is>
-          <t>Saucony London 10K</t>
+          <t>Run in Lyon (10K)</t>
         </is>
       </c>
       <c r="B875" s="5" t="inlineStr">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="D875" s="5" t="inlineStr">
         <is>
-          <t>0:29:33</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E875" s="5" t="inlineStr">
@@ -22365,7 +22365,7 @@
     <row r="876">
       <c r="A876" s="8" t="inlineStr">
         <is>
-          <t>Standard Chartered KL 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B876" s="9" t="inlineStr">
@@ -22374,23 +22374,23 @@
         </is>
       </c>
       <c r="C876" s="9" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D876" s="9" t="inlineStr">
         <is>
-          <t>0:32:26</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E876" s="9" t="inlineStr">
         <is>
-          <t>0:39:23</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="877">
       <c r="A877" s="4" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B877" s="5" t="inlineStr">
@@ -22399,23 +22399,23 @@
         </is>
       </c>
       <c r="C877" s="5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D877" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:41</t>
         </is>
       </c>
       <c r="E877" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:51</t>
         </is>
       </c>
     </row>
     <row r="878">
       <c r="A878" s="8" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Saucony London 10K</t>
         </is>
       </c>
       <c r="B878" s="9" t="inlineStr">
@@ -22424,11 +22424,11 @@
         </is>
       </c>
       <c r="C878" s="9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D878" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:29:33</t>
         </is>
       </c>
       <c r="E878" s="9" t="inlineStr">
@@ -22440,7 +22440,7 @@
     <row r="879">
       <c r="A879" s="4" t="inlineStr">
         <is>
-          <t>Statesman Capitol 10K</t>
+          <t>Standard Chartered KL 10K</t>
         </is>
       </c>
       <c r="B879" s="5" t="inlineStr">
@@ -22453,19 +22453,19 @@
       </c>
       <c r="D879" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:26</t>
         </is>
       </c>
       <c r="E879" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:39:23</t>
         </is>
       </c>
     </row>
     <row r="880">
       <c r="A880" s="8" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B880" s="9" t="inlineStr">
@@ -22490,7 +22490,7 @@
     <row r="881">
       <c r="A881" s="4" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B881" s="5" t="inlineStr">
@@ -22515,7 +22515,7 @@
     <row r="882">
       <c r="A882" s="8" t="inlineStr">
         <is>
-          <t>Transurban Bridge to Brisbane</t>
+          <t>Statesman Capitol 10K</t>
         </is>
       </c>
       <c r="B882" s="9" t="inlineStr">
@@ -22540,7 +22540,7 @@
     <row r="883">
       <c r="A883" s="4" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B883" s="5" t="inlineStr">
@@ -22565,7 +22565,7 @@
     <row r="884">
       <c r="A884" s="8" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B884" s="9" t="inlineStr">
@@ -22590,7 +22590,7 @@
     <row r="885">
       <c r="A885" s="4" t="inlineStr">
         <is>
-          <t>Ukrop's Monument Avenue 10K</t>
+          <t>Transurban Bridge to Brisbane</t>
         </is>
       </c>
       <c r="B885" s="5" t="inlineStr">
@@ -22615,7 +22615,7 @@
     <row r="886">
       <c r="A886" s="8" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Ukrop's Monument Avenue 10K</t>
         </is>
       </c>
       <c r="B886" s="9" t="inlineStr">
@@ -22640,7 +22640,7 @@
     <row r="887">
       <c r="A887" s="4" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Ukrop's Monument Avenue 10K</t>
         </is>
       </c>
       <c r="B887" s="5" t="inlineStr">
@@ -22665,7 +22665,7 @@
     <row r="888">
       <c r="A888" s="8" t="inlineStr">
         <is>
-          <t>Vancouver Sun Run</t>
+          <t>Ukrop's Monument Avenue 10K</t>
         </is>
       </c>
       <c r="B888" s="9" t="inlineStr">
@@ -22678,19 +22678,19 @@
       </c>
       <c r="D888" s="9" t="inlineStr">
         <is>
-          <t>0:28:09</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E888" s="9" t="inlineStr">
         <is>
-          <t>0:32:54</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="889">
       <c r="A889" s="4" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Vancouver Sun Run</t>
         </is>
       </c>
       <c r="B889" s="5" t="inlineStr">
@@ -22715,7 +22715,7 @@
     <row r="890">
       <c r="A890" s="8" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Vancouver Sun Run</t>
         </is>
       </c>
       <c r="B890" s="9" t="inlineStr">
@@ -22728,19 +22728,19 @@
       </c>
       <c r="D890" s="9" t="inlineStr">
         <is>
-          <t>0:29:14</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E890" s="9" t="inlineStr">
         <is>
-          <t>0:31:36</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="891">
       <c r="A891" s="4" t="inlineStr">
         <is>
-          <t>Vitality London 10,000</t>
+          <t>Vancouver Sun Run</t>
         </is>
       </c>
       <c r="B891" s="5" t="inlineStr">
@@ -22753,28 +22753,28 @@
       </c>
       <c r="D891" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:28:09</t>
         </is>
       </c>
       <c r="E891" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:32:54</t>
         </is>
       </c>
     </row>
     <row r="892">
       <c r="A892" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great Birmingham Run</t>
+          <t>Vitality London 10,000</t>
         </is>
       </c>
       <c r="B892" s="9" t="inlineStr">
         <is>
-          <t>SEMI</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="C892" s="9" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D892" s="9" t="inlineStr">
         <is>
@@ -22790,37 +22790,37 @@
     <row r="893">
       <c r="A893" s="4" t="inlineStr">
         <is>
-          <t>AJ Bell Great South Run</t>
+          <t>Vitality London 10,000</t>
         </is>
       </c>
       <c r="B893" s="5" t="inlineStr">
         <is>
-          <t>AUTRE</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="C893" s="5" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D893" s="5" t="inlineStr">
         <is>
-          <t>0:47:19</t>
+          <t>0:29:14</t>
         </is>
       </c>
       <c r="E893" s="5" t="inlineStr">
         <is>
-          <t>0:50:42</t>
+          <t>0:31:36</t>
         </is>
       </c>
     </row>
     <row r="894">
       <c r="A894" s="8" t="inlineStr">
         <is>
-          <t>AJ Bell Great South Run</t>
+          <t>Vitality London 10,000</t>
         </is>
       </c>
       <c r="B894" s="9" t="inlineStr">
         <is>
-          <t>AUTRE</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="C894" s="9" t="n">
@@ -22840,7 +22840,7 @@
     <row r="895">
       <c r="A895" s="4" t="inlineStr">
         <is>
-          <t>Army Ten Miler</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B895" s="5" t="inlineStr">
@@ -22849,11 +22849,11 @@
         </is>
       </c>
       <c r="C895" s="5" t="n">
-        <v>2025</v>
+        <v>2013</v>
       </c>
       <c r="D895" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:21</t>
         </is>
       </c>
       <c r="E895" s="5" t="inlineStr">
@@ -22865,7 +22865,7 @@
     <row r="896">
       <c r="A896" s="8" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B896" s="9" t="inlineStr">
@@ -22874,23 +22874,23 @@
         </is>
       </c>
       <c r="C896" s="9" t="n">
-        <v>2005</v>
+        <v>2014</v>
       </c>
       <c r="D896" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:05</t>
         </is>
       </c>
       <c r="E896" s="9" t="inlineStr">
         <is>
-          <t>0:38:22</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="897">
       <c r="A897" s="4" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B897" s="5" t="inlineStr">
@@ -22899,11 +22899,11 @@
         </is>
       </c>
       <c r="C897" s="5" t="n">
-        <v>2009</v>
+        <v>2015</v>
       </c>
       <c r="D897" s="5" t="inlineStr">
         <is>
-          <t>0:33:31</t>
+          <t>1:01:47</t>
         </is>
       </c>
       <c r="E897" s="5" t="inlineStr">
@@ -22915,7 +22915,7 @@
     <row r="898">
       <c r="A898" s="8" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B898" s="9" t="inlineStr">
@@ -22924,23 +22924,23 @@
         </is>
       </c>
       <c r="C898" s="9" t="n">
-        <v>2010</v>
+        <v>2016</v>
       </c>
       <c r="D898" s="9" t="inlineStr">
         <is>
-          <t>0:34:15</t>
+          <t>1:02:07</t>
         </is>
       </c>
       <c r="E898" s="9" t="inlineStr">
         <is>
-          <t>0:38:07</t>
+          <t>1:13:51</t>
         </is>
       </c>
     </row>
     <row r="899">
       <c r="A899" s="4" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B899" s="5" t="inlineStr">
@@ -22949,23 +22949,23 @@
         </is>
       </c>
       <c r="C899" s="5" t="n">
-        <v>2012</v>
+        <v>2017</v>
       </c>
       <c r="D899" s="5" t="inlineStr">
         <is>
-          <t>0:34:40</t>
+          <t>1:00:37</t>
         </is>
       </c>
       <c r="E899" s="5" t="inlineStr">
         <is>
-          <t>0:39:02</t>
+          <t>1:13:42</t>
         </is>
       </c>
     </row>
     <row r="900">
       <c r="A900" s="8" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B900" s="9" t="inlineStr">
@@ -22974,23 +22974,23 @@
         </is>
       </c>
       <c r="C900" s="9" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="D900" s="9" t="inlineStr">
         <is>
-          <t>0:35:01</t>
+          <t>1:02:56</t>
         </is>
       </c>
       <c r="E900" s="9" t="inlineStr">
         <is>
-          <t>0:39:28</t>
+          <t>1:14:38</t>
         </is>
       </c>
     </row>
     <row r="901">
       <c r="A901" s="4" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B901" s="5" t="inlineStr">
@@ -22999,23 +22999,23 @@
         </is>
       </c>
       <c r="C901" s="5" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D901" s="5" t="inlineStr">
         <is>
-          <t>0:36:10</t>
+          <t>1:00:34</t>
         </is>
       </c>
       <c r="E901" s="5" t="inlineStr">
         <is>
-          <t>0:42:05</t>
+          <t>1:13:04</t>
         </is>
       </c>
     </row>
     <row r="902">
       <c r="A902" s="8" t="inlineStr">
         <is>
-          <t>Bay to Breakers</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B902" s="9" t="inlineStr">
@@ -23024,23 +23024,23 @@
         </is>
       </c>
       <c r="C902" s="9" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D902" s="9" t="inlineStr">
         <is>
-          <t>0:37:02</t>
+          <t>0:59:31</t>
         </is>
       </c>
       <c r="E902" s="9" t="inlineStr">
         <is>
-          <t>0:43:48</t>
+          <t>1:09:50</t>
         </is>
       </c>
     </row>
     <row r="903">
       <c r="A903" s="4" t="inlineStr">
         <is>
-          <t>Boilermaker Road Race</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B903" s="5" t="inlineStr">
@@ -23049,23 +23049,23 @@
         </is>
       </c>
       <c r="C903" s="5" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="D903" s="5" t="inlineStr">
         <is>
-          <t>0:42:44</t>
+          <t>1:00:01</t>
         </is>
       </c>
       <c r="E903" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:11:11</t>
         </is>
       </c>
     </row>
     <row r="904">
       <c r="A904" s="8" t="inlineStr">
         <is>
-          <t>Broad Street Run</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B904" s="9" t="inlineStr">
@@ -23074,23 +23074,23 @@
         </is>
       </c>
       <c r="C904" s="9" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D904" s="9" t="inlineStr">
         <is>
-          <t>0:46:13</t>
+          <t>1:00:15</t>
         </is>
       </c>
       <c r="E904" s="9" t="inlineStr">
         <is>
-          <t>0:54:01</t>
+          <t>1:10:44</t>
         </is>
       </c>
     </row>
     <row r="905">
       <c r="A905" s="4" t="inlineStr">
         <is>
-          <t>City2Surf</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B905" s="5" t="inlineStr">
@@ -23103,19 +23103,19 @@
       </c>
       <c r="D905" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:57</t>
         </is>
       </c>
       <c r="E905" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1:10:56</t>
         </is>
       </c>
     </row>
     <row r="906">
       <c r="A906" s="8" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>20KM de Bruxelles</t>
         </is>
       </c>
       <c r="B906" s="9" t="inlineStr">
@@ -23124,32 +23124,32 @@
         </is>
       </c>
       <c r="C906" s="9" t="n">
-        <v>2009</v>
+        <v>2025</v>
       </c>
       <c r="D906" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:59:26</t>
         </is>
       </c>
       <c r="E906" s="9" t="inlineStr">
         <is>
-          <t>0:50:39</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="907">
       <c r="A907" s="4" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>AJ Bell Great Birmingham Run</t>
         </is>
       </c>
       <c r="B907" s="5" t="inlineStr">
         <is>
-          <t>AUTRE</t>
+          <t>SEMI</t>
         </is>
       </c>
       <c r="C907" s="5" t="n">
-        <v>2010</v>
+        <v>2025</v>
       </c>
       <c r="D907" s="5" t="inlineStr">
         <is>
@@ -23158,14 +23158,14 @@
       </c>
       <c r="E907" s="5" t="inlineStr">
         <is>
-          <t>0:51:30</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="908">
       <c r="A908" s="8" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>AJ Bell Great South Run</t>
         </is>
       </c>
       <c r="B908" s="9" t="inlineStr">
@@ -23174,23 +23174,23 @@
         </is>
       </c>
       <c r="C908" s="9" t="n">
-        <v>2011</v>
+        <v>2021</v>
       </c>
       <c r="D908" s="9" t="inlineStr">
         <is>
-          <t>0:44:27</t>
+          <t>0:47:19</t>
         </is>
       </c>
       <c r="E908" s="9" t="inlineStr">
         <is>
-          <t>0:51:57</t>
+          <t>0:50:42</t>
         </is>
       </c>
     </row>
     <row r="909">
       <c r="A909" s="4" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>AJ Bell Great South Run</t>
         </is>
       </c>
       <c r="B909" s="5" t="inlineStr">
@@ -23199,23 +23199,23 @@
         </is>
       </c>
       <c r="C909" s="5" t="n">
-        <v>2012</v>
+        <v>2025</v>
       </c>
       <c r="D909" s="5" t="inlineStr">
         <is>
-          <t>0:44:48</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E909" s="5" t="inlineStr">
         <is>
-          <t>0:51:42</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="910">
       <c r="A910" s="8" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>Army Ten Miler</t>
         </is>
       </c>
       <c r="B910" s="9" t="inlineStr">
@@ -23224,23 +23224,23 @@
         </is>
       </c>
       <c r="C910" s="9" t="n">
-        <v>2013</v>
+        <v>2025</v>
       </c>
       <c r="D910" s="9" t="inlineStr">
         <is>
-          <t>0:45:28</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E910" s="9" t="inlineStr">
         <is>
-          <t>0:51:33</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="911">
       <c r="A911" s="4" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>Baloise Antwerp 10 miles</t>
         </is>
       </c>
       <c r="B911" s="5" t="inlineStr">
@@ -23249,23 +23249,23 @@
         </is>
       </c>
       <c r="C911" s="5" t="n">
-        <v>2014</v>
+        <v>2022</v>
       </c>
       <c r="D911" s="5" t="inlineStr">
         <is>
-          <t>0:45:45</t>
+          <t>0:48:48</t>
         </is>
       </c>
       <c r="E911" s="5" t="inlineStr">
         <is>
-          <t>0:53:09</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="912">
       <c r="A912" s="8" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>Baloise Antwerp 10 miles</t>
         </is>
       </c>
       <c r="B912" s="9" t="inlineStr">
@@ -23274,23 +23274,23 @@
         </is>
       </c>
       <c r="C912" s="9" t="n">
-        <v>2019</v>
+        <v>2023</v>
       </c>
       <c r="D912" s="9" t="inlineStr">
         <is>
-          <t>0:45:15</t>
+          <t>0:47:50</t>
         </is>
       </c>
       <c r="E912" s="9" t="inlineStr">
         <is>
-          <t>0:50:45</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="913">
       <c r="A913" s="4" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>Baloise Antwerp 10 miles</t>
         </is>
       </c>
       <c r="B913" s="5" t="inlineStr">
@@ -23299,23 +23299,23 @@
         </is>
       </c>
       <c r="C913" s="5" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="D913" s="5" t="inlineStr">
         <is>
-          <t>0:49:00</t>
+          <t>0:47:21</t>
         </is>
       </c>
       <c r="E913" s="5" t="inlineStr">
         <is>
-          <t>0:55:44</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="914">
       <c r="A914" s="8" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>Bay to Breakers</t>
         </is>
       </c>
       <c r="B914" s="9" t="inlineStr">
@@ -23324,23 +23324,23 @@
         </is>
       </c>
       <c r="C914" s="9" t="n">
-        <v>2024</v>
+        <v>2005</v>
       </c>
       <c r="D914" s="9" t="inlineStr">
         <is>
-          <t>0:44:51</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E914" s="9" t="inlineStr">
         <is>
-          <t>0:51:15</t>
+          <t>0:38:22</t>
         </is>
       </c>
     </row>
     <row r="915">
       <c r="A915" s="4" t="inlineStr">
         <is>
-          <t>Dam tot Damloop</t>
+          <t>Bay to Breakers</t>
         </is>
       </c>
       <c r="B915" s="5" t="inlineStr">
@@ -23349,23 +23349,23 @@
         </is>
       </c>
       <c r="C915" s="5" t="n">
-        <v>2025</v>
+        <v>2009</v>
       </c>
       <c r="D915" s="5" t="inlineStr">
         <is>
-          <t>0:46:07</t>
+          <t>0:33:31</t>
         </is>
       </c>
       <c r="E915" s="5" t="inlineStr">
         <is>
-          <t>0:50:51</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="916">
       <c r="A916" s="8" t="inlineStr">
         <is>
-          <t>Falmouth Road Race</t>
+          <t>Bay to Breakers</t>
         </is>
       </c>
       <c r="B916" s="9" t="inlineStr">
@@ -23374,48 +23374,48 @@
         </is>
       </c>
       <c r="C916" s="9" t="n">
-        <v>2025</v>
+        <v>2010</v>
       </c>
       <c r="D916" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:34:15</t>
         </is>
       </c>
       <c r="E916" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:38:07</t>
         </is>
       </c>
     </row>
     <row r="917">
       <c r="A917" s="4" t="inlineStr">
         <is>
-          <t>Great Scottish Run</t>
+          <t>Bay to Breakers</t>
         </is>
       </c>
       <c r="B917" s="5" t="inlineStr">
         <is>
-          <t>SEMI</t>
+          <t>AUTRE</t>
         </is>
       </c>
       <c r="C917" s="5" t="n">
-        <v>2025</v>
+        <v>2012</v>
       </c>
       <c r="D917" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:34:40</t>
         </is>
       </c>
       <c r="E917" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:39:02</t>
         </is>
       </c>
     </row>
     <row r="918">
       <c r="A918" s="8" t="inlineStr">
         <is>
-          <t>Lilac Bloomsday Run</t>
+          <t>Bay to Breakers</t>
         </is>
       </c>
       <c r="B918" s="9" t="inlineStr">
@@ -23424,46 +23424,496 @@
         </is>
       </c>
       <c r="C918" s="9" t="n">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="D918" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:35:01</t>
         </is>
       </c>
       <c r="E918" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0:39:28</t>
         </is>
       </c>
     </row>
     <row r="919">
       <c r="A919" s="4" t="inlineStr">
         <is>
+          <t>Bay to Breakers</t>
+        </is>
+      </c>
+      <c r="B919" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C919" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D919" s="5" t="inlineStr">
+        <is>
+          <t>0:36:10</t>
+        </is>
+      </c>
+      <c r="E919" s="5" t="inlineStr">
+        <is>
+          <t>0:42:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="8" t="inlineStr">
+        <is>
+          <t>Bay to Breakers</t>
+        </is>
+      </c>
+      <c r="B920" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C920" s="9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D920" s="9" t="inlineStr">
+        <is>
+          <t>0:37:02</t>
+        </is>
+      </c>
+      <c r="E920" s="9" t="inlineStr">
+        <is>
+          <t>0:43:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="4" t="inlineStr">
+        <is>
+          <t>Boilermaker Road Race</t>
+        </is>
+      </c>
+      <c r="B921" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C921" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D921" s="5" t="inlineStr">
+        <is>
+          <t>0:42:44</t>
+        </is>
+      </c>
+      <c r="E921" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="8" t="inlineStr">
+        <is>
+          <t>Broad Street Run</t>
+        </is>
+      </c>
+      <c r="B922" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C922" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D922" s="9" t="inlineStr">
+        <is>
+          <t>0:46:13</t>
+        </is>
+      </c>
+      <c r="E922" s="9" t="inlineStr">
+        <is>
+          <t>0:54:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="4" t="inlineStr">
+        <is>
+          <t>City2Surf</t>
+        </is>
+      </c>
+      <c r="B923" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C923" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D923" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E923" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="8" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B924" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C924" s="9" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D924" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E924" s="9" t="inlineStr">
+        <is>
+          <t>0:50:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="4" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B925" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C925" s="5" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D925" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E925" s="5" t="inlineStr">
+        <is>
+          <t>0:51:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="8" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B926" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C926" s="9" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D926" s="9" t="inlineStr">
+        <is>
+          <t>0:44:27</t>
+        </is>
+      </c>
+      <c r="E926" s="9" t="inlineStr">
+        <is>
+          <t>0:51:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="4" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B927" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C927" s="5" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D927" s="5" t="inlineStr">
+        <is>
+          <t>0:44:48</t>
+        </is>
+      </c>
+      <c r="E927" s="5" t="inlineStr">
+        <is>
+          <t>0:51:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="8" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B928" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C928" s="9" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D928" s="9" t="inlineStr">
+        <is>
+          <t>0:45:28</t>
+        </is>
+      </c>
+      <c r="E928" s="9" t="inlineStr">
+        <is>
+          <t>0:51:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="4" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B929" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C929" s="5" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D929" s="5" t="inlineStr">
+        <is>
+          <t>0:45:45</t>
+        </is>
+      </c>
+      <c r="E929" s="5" t="inlineStr">
+        <is>
+          <t>0:53:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="8" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B930" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C930" s="9" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D930" s="9" t="inlineStr">
+        <is>
+          <t>0:45:15</t>
+        </is>
+      </c>
+      <c r="E930" s="9" t="inlineStr">
+        <is>
+          <t>0:50:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="4" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B931" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C931" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D931" s="5" t="inlineStr">
+        <is>
+          <t>0:49:00</t>
+        </is>
+      </c>
+      <c r="E931" s="5" t="inlineStr">
+        <is>
+          <t>0:55:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="8" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B932" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C932" s="9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D932" s="9" t="inlineStr">
+        <is>
+          <t>0:44:51</t>
+        </is>
+      </c>
+      <c r="E932" s="9" t="inlineStr">
+        <is>
+          <t>0:51:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="4" t="inlineStr">
+        <is>
+          <t>Dam tot Damloop</t>
+        </is>
+      </c>
+      <c r="B933" s="5" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C933" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D933" s="5" t="inlineStr">
+        <is>
+          <t>0:46:07</t>
+        </is>
+      </c>
+      <c r="E933" s="5" t="inlineStr">
+        <is>
+          <t>0:50:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="8" t="inlineStr">
+        <is>
+          <t>Falmouth Road Race</t>
+        </is>
+      </c>
+      <c r="B934" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C934" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D934" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E934" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="4" t="inlineStr">
+        <is>
+          <t>Great Scottish Run</t>
+        </is>
+      </c>
+      <c r="B935" s="5" t="inlineStr">
+        <is>
+          <t>SEMI</t>
+        </is>
+      </c>
+      <c r="C935" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D935" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E935" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="8" t="inlineStr">
+        <is>
+          <t>Lilac Bloomsday Run</t>
+        </is>
+      </c>
+      <c r="B936" s="9" t="inlineStr">
+        <is>
+          <t>AUTRE</t>
+        </is>
+      </c>
+      <c r="C936" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D936" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E936" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="4" t="inlineStr">
+        <is>
           <t>Manchester Road Race</t>
         </is>
       </c>
-      <c r="B919" s="5" t="inlineStr">
+      <c r="B937" s="5" t="inlineStr">
         <is>
           <t>AUTRE</t>
         </is>
       </c>
-      <c r="C919" s="5" t="n">
+      <c r="C937" s="5" t="n">
         <v>2024</v>
       </c>
-      <c r="D919" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E919" s="5" t="inlineStr">
+      <c r="D937" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E937" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E919"/>
+  <autoFilter ref="A1:E937"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>